<commit_message>
radar 2026-08-30: +0 novas, 0 atualizadas, 0 snapshots
</commit_message>
<xml_diff>
--- a/Radar/radar-low-ticket.xlsx
+++ b/Radar/radar-low-ticket.xlsx
@@ -16,7 +16,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Resumo por nicho'!$A$1:$G$3</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Varredura'!$A$1:$D$7</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Achados'!$A$1:$L$8</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Achados'!$A$1:$L$5</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -736,7 +736,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L8"/>
+  <dimension ref="A1:L5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -818,14 +818,14 @@
     <row r="2">
       <c r="A2" s="12" t="inlineStr">
         <is>
+          <t>stalkeia</t>
+        </is>
+      </c>
+      <c r="B2" s="12" t="inlineStr">
+        <is>
           <t>Stalkeia</t>
         </is>
       </c>
-      <c r="B2" s="12" t="inlineStr">
-        <is>
-          <t>Stalkeia.ai</t>
-        </is>
-      </c>
       <c r="C2" s="12" t="inlineStr">
         <is>
           <t>marca</t>
@@ -843,45 +843,41 @@
       </c>
       <c r="F2" s="12" t="inlineStr">
         <is>
-          <t>quente</t>
+          <t>fria</t>
         </is>
       </c>
       <c r="G2" s="12" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H2" s="12" t="inlineStr">
         <is>
-          <t>R$ 47-87</t>
+          <t>R$ 37,00</t>
         </is>
       </c>
       <c r="I2" s="12" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-08-30</t>
         </is>
       </c>
       <c r="J2" s="12" t="n">
         <v>1</v>
       </c>
-      <c r="K2" s="12" t="inlineStr">
-        <is>
-          <t>App de espionar WhatsApp/Instagram. Grafias: Stalkeia.com, Stalkeia App, IA STALKER. Cobra créditos extras para liberar resultado. Três menções em 25/08-26/08 com valores R$ 47 e R$ 87.</t>
-        </is>
-      </c>
+      <c r="K2" s="12" t="inlineStr"/>
       <c r="L2" s="12" t="inlineStr">
         <is>
-          <t>https://www.reclameaqui.com.br/perfectpay/cobranca-de-taxa-adicional-nao-combinada-e-falta-de-acesso-ao-produto-comprado__chfFQTX8pupMWB5/</t>
+          <t>https://www.reclameaqui.com.br/perfectpay/propaganda-enganosa-do-aplicativo-stalkeia-app-e-solicitacao-de-reembolso_zrIGWUSWcSp7p5Xp/</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="12" t="inlineStr">
         <is>
-          <t>hqflix</t>
+          <t>spygram</t>
         </is>
       </c>
       <c r="B3" s="12" t="inlineStr">
         <is>
-          <t>hqflix</t>
+          <t>Spygram</t>
         </is>
       </c>
       <c r="C3" s="12" t="inlineStr">
@@ -891,12 +887,12 @@
       </c>
       <c r="D3" s="12" t="inlineStr">
         <is>
-          <t>Cakto</t>
+          <t>PerfectPay</t>
         </is>
       </c>
       <c r="E3" s="12" t="inlineStr">
         <is>
-          <t>Streaming e entretenimento</t>
+          <t>Espionagem e rastreamento</t>
         </is>
       </c>
       <c r="F3" s="12" t="inlineStr">
@@ -907,40 +903,40 @@
       <c r="G3" s="12" t="n">
         <v>1</v>
       </c>
-      <c r="H3" s="12" t="inlineStr"/>
+      <c r="H3" s="12" t="inlineStr">
+        <is>
+          <t>R$ 49,80</t>
+        </is>
+      </c>
       <c r="I3" s="12" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-08-30</t>
         </is>
       </c>
       <c r="J3" s="12" t="n">
         <v>1</v>
       </c>
-      <c r="K3" s="12" t="inlineStr">
-        <is>
-          <t>Serviço de streaming anunciado como acesso vitalício. Comprador de 21/11/2025 não consegue mais acessar. Solicita estorno.</t>
-        </is>
-      </c>
+      <c r="K3" s="12" t="inlineStr"/>
       <c r="L3" s="12" t="inlineStr">
         <is>
-          <t>https://www.reclameaqui.com.br/cakto-pay/usuario-solicita-estorno-por-nao-conseguir-mais-acessar-o-servico-hqflix-que-foi-anunciado-como-acesso-vitalicio_7zfD-D4s6GauY3fc/</t>
+          <t>https://www.reclameaqui.com.br/perfectpay/usuario-pagou-por-app-de-monitoramento-falso-e-nao-recebeu-acesso-a-nada-solicita-reembolso_h9AXG_wRQFTAEB9J/</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="12" t="inlineStr">
         <is>
-          <t>freelancer imediato</t>
+          <t>comprado. gostaria do reembolso assim que</t>
         </is>
       </c>
       <c r="B4" s="12" t="inlineStr">
         <is>
-          <t>PLANO FREELANCER IMEDIATO</t>
+          <t>comprado. Gostaria do reembolso assim que</t>
         </is>
       </c>
       <c r="C4" s="12" t="inlineStr">
         <is>
-          <t>marca</t>
+          <t>angulo</t>
         </is>
       </c>
       <c r="D4" s="12" t="inlineStr">
@@ -950,7 +946,7 @@
       </c>
       <c r="E4" s="12" t="inlineStr">
         <is>
-          <t>Ganhar dinheiro online / trabalho remoto</t>
+          <t>Ferramentas de IA / Produtividade</t>
         </is>
       </c>
       <c r="F4" s="12" t="inlineStr">
@@ -961,39 +957,31 @@
       <c r="G4" s="12" t="n">
         <v>1</v>
       </c>
-      <c r="H4" s="12" t="inlineStr">
-        <is>
-          <t>R$ 11 + R$ 30 upsell</t>
-        </is>
-      </c>
+      <c r="H4" s="12" t="inlineStr"/>
       <c r="I4" s="12" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-08-30</t>
         </is>
       </c>
       <c r="J4" s="12" t="n">
         <v>1</v>
       </c>
-      <c r="K4" s="12" t="inlineStr">
-        <is>
-          <t>Plano vendido pela equipe Cakto por R$ 11 para acessar sites de trabalho remoto. Após pagamento, exige R$ 30 adicional para liberar acesso. Mecânica de taxa para desbloquear.</t>
-        </is>
-      </c>
+      <c r="K4" s="12" t="inlineStr"/>
       <c r="L4" s="12" t="inlineStr">
         <is>
-          <t>https://www.reclameaqui.com.br/cakto-pay/plano-freelancer-imediato-pagamento-adicional-exigido-apos-compra-inicial-para-liberacao-de-acesso_Aa7b4b27tHVPApDH/</t>
+          <t>https://www.reclameaqui.com.br/cakto-pay/pagamento-via-pix-nao-resultou-na-entrega-do-produto-solicitacao-de-reembolso-por-possivel-editado-pelo-reclame-aqui_cbUdm8Fq5-5oanwH/</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="12" t="inlineStr">
         <is>
-          <t>pagamento nao recebido cakto</t>
+          <t>curso online</t>
         </is>
       </c>
       <c r="B5" s="12" t="inlineStr">
         <is>
-          <t>Pagamentos não recebidos (ângulo)</t>
+          <t>curso online</t>
         </is>
       </c>
       <c r="C5" s="12" t="inlineStr">
@@ -1008,7 +996,7 @@
       </c>
       <c r="E5" s="12" t="inlineStr">
         <is>
-          <t>Serviços financeiros / Pix</t>
+          <t>Ferramentas de IA / Produtividade</t>
         </is>
       </c>
       <c r="F5" s="12" t="inlineStr">
@@ -1019,198 +1007,24 @@
       <c r="G5" s="12" t="n">
         <v>1</v>
       </c>
-      <c r="H5" s="12" t="inlineStr">
-        <is>
-          <t>R$ 13,89 + R$ 38,89</t>
-        </is>
-      </c>
+      <c r="H5" s="12" t="inlineStr"/>
       <c r="I5" s="12" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-08-30</t>
         </is>
       </c>
       <c r="J5" s="12" t="n">
         <v>1</v>
       </c>
-      <c r="K5" s="12" t="inlineStr">
-        <is>
-          <t>Cliente alega ter feito pagamentos via Cakto Pay (R$ 13,89 e R$ 38,89) e não ter recebido o serviço. Padrão de cobrança sem entrega.</t>
-        </is>
-      </c>
+      <c r="K5" s="12" t="inlineStr"/>
       <c r="L5" s="12" t="inlineStr">
         <is>
-          <t>https://www.reclameaqui.com.br/cakto-pay/cliente-alega-ter-sido-editado-pelo-reclame-aqui-pela-cakto-pay-apos-solicitacao-de-pagamento-nao-recebido_iGkp9DgcxElv0_2Y/</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="12" t="inlineStr">
-        <is>
-          <t>reembolso cakto dificuldade</t>
-        </is>
-      </c>
-      <c r="B6" s="12" t="inlineStr">
-        <is>
-          <t>Dificuldade de reembolso Cakto (ângulo)</t>
-        </is>
-      </c>
-      <c r="C6" s="12" t="inlineStr">
-        <is>
-          <t>angulo</t>
-        </is>
-      </c>
-      <c r="D6" s="12" t="inlineStr">
-        <is>
-          <t>Cakto</t>
-        </is>
-      </c>
-      <c r="E6" s="12" t="inlineStr">
-        <is>
-          <t>Infoprodutos - suporte e reembolso</t>
-        </is>
-      </c>
-      <c r="F6" s="12" t="inlineStr">
-        <is>
-          <t>fria</t>
-        </is>
-      </c>
-      <c r="G6" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="H6" s="12" t="inlineStr"/>
-      <c r="I6" s="12" t="inlineStr">
-        <is>
-          <t>2026-08-26</t>
-        </is>
-      </c>
-      <c r="J6" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="K6" s="12" t="inlineStr">
-        <is>
-          <t>Comprador pediu reembolso em menos de 4 dias, não obteve resposta do produtor nem suporte da Cakto. Indica falha no fluxo de reembolso da plataforma.</t>
-        </is>
-      </c>
-      <c r="L6" s="12" t="inlineStr">
-        <is>
-          <t>https://www.reclameaqui.com.br/cakto-pay/reclamacao-sobre-falta-de-resposta-e-dificuldade-de-reembolso-na-cakto_jiJdywNvdI1eyqGx/</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="12" t="inlineStr">
-        <is>
-          <t>conta digital cakto validacao falha</t>
-        </is>
-      </c>
-      <c r="B7" s="12" t="inlineStr">
-        <is>
-          <t>Falha validação Conta Digital Cakto - produtor (ângulo)</t>
-        </is>
-      </c>
-      <c r="C7" s="12" t="inlineStr">
-        <is>
-          <t>angulo</t>
-        </is>
-      </c>
-      <c r="D7" s="12" t="inlineStr">
-        <is>
-          <t>Cakto</t>
-        </is>
-      </c>
-      <c r="E7" s="12" t="inlineStr">
-        <is>
-          <t>Serviços financeiros / conta digital</t>
-        </is>
-      </c>
-      <c r="F7" s="12" t="inlineStr">
-        <is>
-          <t>fria</t>
-        </is>
-      </c>
-      <c r="G7" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="H7" s="12" t="inlineStr">
-        <is>
-          <t>R$ 1.100+ retidos</t>
-        </is>
-      </c>
-      <c r="I7" s="12" t="inlineStr">
-        <is>
-          <t>2026-08-26</t>
-        </is>
-      </c>
-      <c r="J7" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="K7" s="12" t="inlineStr">
-        <is>
-          <t>Produtor com vendas ativas não consegue transferir saldo (R$ 1.100+) por falha na validação da Conta Digital Cakto. Suporte lento, 15+ dias sem resolução. Travando operação de tráfego pago.</t>
-        </is>
-      </c>
-      <c r="L7" s="12" t="inlineStr">
-        <is>
-          <t>https://www.reclameaqui.com.br/cakto-pay/produtor-da-cakto-nao-consegue-transferir-saldo-de-vendas-devido-a-falha-na-validacao-da-conta-digital_4DnOrKwoT1hMSEch/</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="12" t="inlineStr">
-        <is>
-          <t>reembolso perfectpay recusa</t>
-        </is>
-      </c>
-      <c r="B8" s="12" t="inlineStr">
-        <is>
-          <t>Recusa reembolso PerfectPay (ângulo)</t>
-        </is>
-      </c>
-      <c r="C8" s="12" t="inlineStr">
-        <is>
-          <t>angulo</t>
-        </is>
-      </c>
-      <c r="D8" s="12" t="inlineStr">
-        <is>
-          <t>PerfectPay</t>
-        </is>
-      </c>
-      <c r="E8" s="12" t="inlineStr">
-        <is>
-          <t>Infoprodutos - suporte e reembolso</t>
-        </is>
-      </c>
-      <c r="F8" s="12" t="inlineStr">
-        <is>
-          <t>fria</t>
-        </is>
-      </c>
-      <c r="G8" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="H8" s="12" t="inlineStr"/>
-      <c r="I8" s="12" t="inlineStr">
-        <is>
-          <t>2026-08-26</t>
-        </is>
-      </c>
-      <c r="J8" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="K8" s="12" t="inlineStr">
-        <is>
-          <t>Comprador solicita reembolso horas após compra, envia provas (PIX, email cancelamento, WhatsApp inativo). PerfectPay responde com mensagens robóticas genéricas pedindo mesmas infos já anexadas. Recusa intervir.</t>
-        </is>
-      </c>
-      <c r="L8" s="12" t="inlineStr">
-        <is>
-          <t>https://www.reclameaqui.com.br/perfectpay/reclamacao-sobre-recusa-de-reembolso-e-atendimento-generico-pela-perfect-pay_BFp4AxOI5U-r8e8Q/</t>
+          <t>https://www.reclameaqui.com.br/cakto-pay/curso-online-nao-entregue-apos-pagamento-com-falha-na-comunicacao-e-solicitacao-de-estorno_-bekag5hY78F-1mM/</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L8"/>
+  <autoFilter ref="A1:L5"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1221,7 +1035,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G7"/>
+  <dimension ref="A1:G3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -1273,17 +1087,17 @@
     <row r="2">
       <c r="A2" s="14" t="inlineStr">
         <is>
-          <t>Infoprodutos - suporte e reembolso</t>
+          <t>Espionagem e rastreamento</t>
         </is>
       </c>
       <c r="B2" s="14" t="n">
         <v>2</v>
       </c>
       <c r="C2" s="14" t="n">
+        <v>2</v>
+      </c>
+      <c r="D2" s="14" t="n">
         <v>0</v>
-      </c>
-      <c r="D2" s="14" t="n">
-        <v>2</v>
       </c>
       <c r="E2" s="14" t="n">
         <v>0</v>
@@ -1298,126 +1112,26 @@
     <row r="3">
       <c r="A3" s="14" t="inlineStr">
         <is>
-          <t>Espionagem e rastreamento</t>
+          <t>Ferramentas de IA / Produtividade</t>
         </is>
       </c>
       <c r="B3" s="14" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C3" s="14" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D3" s="14" t="n">
+        <v>2</v>
+      </c>
+      <c r="E3" s="14" t="n">
         <v>0</v>
-      </c>
-      <c r="E3" s="14" t="n">
-        <v>1</v>
       </c>
       <c r="F3" s="14" t="n">
         <v>0</v>
       </c>
       <c r="G3" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="14" t="inlineStr">
-        <is>
-          <t>Streaming e entretenimento</t>
-        </is>
-      </c>
-      <c r="B4" s="14" t="n">
-        <v>1</v>
-      </c>
-      <c r="C4" s="14" t="n">
-        <v>1</v>
-      </c>
-      <c r="D4" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="E4" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="F4" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="G4" s="14" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="14" t="inlineStr">
-        <is>
-          <t>Ganhar dinheiro online / trabalho remoto</t>
-        </is>
-      </c>
-      <c r="B5" s="14" t="n">
-        <v>1</v>
-      </c>
-      <c r="C5" s="14" t="n">
-        <v>1</v>
-      </c>
-      <c r="D5" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="E5" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="F5" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="G5" s="14" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="14" t="inlineStr">
-        <is>
-          <t>Serviços financeiros / Pix</t>
-        </is>
-      </c>
-      <c r="B6" s="14" t="n">
-        <v>1</v>
-      </c>
-      <c r="C6" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="D6" s="14" t="n">
-        <v>1</v>
-      </c>
-      <c r="E6" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="F6" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="G6" s="14" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="14" t="inlineStr">
-        <is>
-          <t>Serviços financeiros / conta digital</t>
-        </is>
-      </c>
-      <c r="B7" s="14" t="n">
-        <v>1</v>
-      </c>
-      <c r="C7" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="D7" s="14" t="n">
-        <v>1</v>
-      </c>
-      <c r="E7" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="F7" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="G7" s="14" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
   </sheetData>
@@ -1431,7 +1145,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C27"/>
+  <dimension ref="A1:C31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -1774,7 +1488,7 @@
         </is>
       </c>
       <c r="C20" s="14" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="21">
@@ -1797,12 +1511,12 @@
     <row r="22">
       <c r="A22" s="14" t="inlineStr">
         <is>
-          <t>conta digital cakto validacao falha</t>
+          <t>comprado. gostaria do reembolso assim que</t>
         </is>
       </c>
       <c r="B22" s="14" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-08-30</t>
         </is>
       </c>
       <c r="C22" s="14" t="n">
@@ -1812,7 +1526,7 @@
     <row r="23">
       <c r="A23" s="14" t="inlineStr">
         <is>
-          <t>freelancer imediato</t>
+          <t>conta digital cakto validacao falha</t>
         </is>
       </c>
       <c r="B23" s="14" t="inlineStr">
@@ -1821,18 +1535,18 @@
         </is>
       </c>
       <c r="C23" s="14" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="14" t="inlineStr">
         <is>
-          <t>hqflix</t>
+          <t>curso online</t>
         </is>
       </c>
       <c r="B24" s="14" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-08-30</t>
         </is>
       </c>
       <c r="C24" s="14" t="n">
@@ -1842,7 +1556,7 @@
     <row r="25">
       <c r="A25" s="14" t="inlineStr">
         <is>
-          <t>pagamento nao recebido cakto</t>
+          <t>freelancer imediato</t>
         </is>
       </c>
       <c r="B25" s="14" t="inlineStr">
@@ -1851,13 +1565,13 @@
         </is>
       </c>
       <c r="C25" s="14" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="14" t="inlineStr">
         <is>
-          <t>reembolso cakto dificuldade</t>
+          <t>hqflix</t>
         </is>
       </c>
       <c r="B26" s="14" t="inlineStr">
@@ -1866,21 +1580,81 @@
         </is>
       </c>
       <c r="C26" s="14" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="14" t="inlineStr">
         <is>
+          <t>pagamento nao recebido cakto</t>
+        </is>
+      </c>
+      <c r="B27" s="14" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+      <c r="C27" s="14" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="14" t="inlineStr">
+        <is>
+          <t>reembolso cakto dificuldade</t>
+        </is>
+      </c>
+      <c r="B28" s="14" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+      <c r="C28" s="14" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="14" t="inlineStr">
+        <is>
           <t>reembolso perfectpay recusa</t>
         </is>
       </c>
-      <c r="B27" s="14" t="inlineStr">
+      <c r="B29" s="14" t="inlineStr">
         <is>
           <t>2026-08-26</t>
         </is>
       </c>
-      <c r="C27" s="14" t="n">
+      <c r="C29" s="14" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="14" t="inlineStr">
+        <is>
+          <t>spygram</t>
+        </is>
+      </c>
+      <c r="B30" s="14" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+      <c r="C30" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="14" t="inlineStr">
+        <is>
+          <t>stalkeia</t>
+        </is>
+      </c>
+      <c r="B31" s="14" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+      <c r="C31" s="14" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
radar 2026-08-31: +0 novas, 0 atualizadas, 0 snapshots
</commit_message>
<xml_diff>
--- a/Radar/radar-low-ticket.xlsx
+++ b/Radar/radar-low-ticket.xlsx
@@ -849,23 +849,19 @@
       <c r="G2" s="12" t="n">
         <v>2</v>
       </c>
-      <c r="H2" s="12" t="inlineStr">
-        <is>
-          <t>R$ 37,00</t>
-        </is>
-      </c>
+      <c r="H2" s="12" t="inlineStr"/>
       <c r="I2" s="12" t="inlineStr">
         <is>
           <t>2026-08-30</t>
         </is>
       </c>
       <c r="J2" s="12" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K2" s="12" t="inlineStr"/>
       <c r="L2" s="12" t="inlineStr">
         <is>
-          <t>https://www.reclameaqui.com.br/perfectpay/propaganda-enganosa-do-aplicativo-stalkeia-app-e-solicitacao-de-reembolso_zrIGWUSWcSp7p5Xp/</t>
+          <t>https://www.reclameaqui.com.br/perfectpay/propaganda-enganosa__4nr816NYlTJmFOB/</t>
         </is>
       </c>
     </row>
@@ -914,7 +910,7 @@
         </is>
       </c>
       <c r="J3" s="12" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K3" s="12" t="inlineStr"/>
       <c r="L3" s="12" t="inlineStr">
@@ -964,7 +960,7 @@
         </is>
       </c>
       <c r="J4" s="12" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K4" s="12" t="inlineStr"/>
       <c r="L4" s="12" t="inlineStr">
@@ -1014,7 +1010,7 @@
         </is>
       </c>
       <c r="J5" s="12" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K5" s="12" t="inlineStr"/>
       <c r="L5" s="12" t="inlineStr">
@@ -1520,7 +1516,7 @@
         </is>
       </c>
       <c r="C22" s="14" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="23">
@@ -1550,7 +1546,7 @@
         </is>
       </c>
       <c r="C24" s="14" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="25">
@@ -1640,7 +1636,7 @@
         </is>
       </c>
       <c r="C30" s="14" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="31">
@@ -1655,7 +1651,7 @@
         </is>
       </c>
       <c r="C31" s="14" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
radar 2026-08-31: +15 novas, 1 atualizadas, 14 snapshots
</commit_message>
<xml_diff>
--- a/Radar/radar-low-ticket.xlsx
+++ b/Radar/radar-low-ticket.xlsx
@@ -16,7 +16,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Resumo por nicho'!$A$1:$G$3</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Varredura'!$A$1:$D$7</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Achados'!$A$1:$L$5</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Achados'!$A$1:$L$4</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -736,7 +736,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L5"/>
+  <dimension ref="A1:L4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -847,33 +847,37 @@
         </is>
       </c>
       <c r="G2" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="H2" s="12" t="inlineStr"/>
+        <v>3</v>
+      </c>
+      <c r="H2" s="12" t="inlineStr">
+        <is>
+          <t>R$ 47,00, R$ 87,00</t>
+        </is>
+      </c>
       <c r="I2" s="12" t="inlineStr">
         <is>
           <t>2026-08-30</t>
         </is>
       </c>
       <c r="J2" s="12" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K2" s="12" t="inlineStr"/>
       <c r="L2" s="12" t="inlineStr">
         <is>
-          <t>https://www.reclameaqui.com.br/perfectpay/propaganda-enganosa-do-aplicativo-stalkeia-app-e-solicitacao-de-reembolso_zrIGWUSWcSp7p5Xp/</t>
+          <t>https://www.reclameaqui.com.br/perfectpay/cobranca-de-taxa-adicional-nao-combinada-e-falta-de-acesso-ao-produto-comprado__chfFQTX8pupMWB5/</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="12" t="inlineStr">
         <is>
-          <t>spygram</t>
+          <t>hqflix</t>
         </is>
       </c>
       <c r="B3" s="12" t="inlineStr">
         <is>
-          <t>Spygram</t>
+          <t>hqflix</t>
         </is>
       </c>
       <c r="C3" s="12" t="inlineStr">
@@ -883,12 +887,12 @@
       </c>
       <c r="D3" s="12" t="inlineStr">
         <is>
-          <t>PerfectPay</t>
+          <t>Cakto</t>
         </is>
       </c>
       <c r="E3" s="12" t="inlineStr">
         <is>
-          <t>Espionagem e rastreamento</t>
+          <t>Streaming e entretenimento</t>
         </is>
       </c>
       <c r="F3" s="12" t="inlineStr">
@@ -899,40 +903,36 @@
       <c r="G3" s="12" t="n">
         <v>1</v>
       </c>
-      <c r="H3" s="12" t="inlineStr">
-        <is>
-          <t>R$ 49,80</t>
-        </is>
-      </c>
+      <c r="H3" s="12" t="inlineStr"/>
       <c r="I3" s="12" t="inlineStr">
         <is>
-          <t>2026-08-30</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="J3" s="12" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K3" s="12" t="inlineStr"/>
       <c r="L3" s="12" t="inlineStr">
         <is>
-          <t>https://www.reclameaqui.com.br/perfectpay/usuario-pagou-por-app-de-monitoramento-falso-e-nao-recebeu-acesso-a-nada-solicita-reembolso_h9AXG_wRQFTAEB9J/</t>
+          <t>https://www.reclameaqui.com.br/cakto-pay/usuario-solicita-estorno-por-nao-conseguir-mais-acessar-o-servico-hqflix-que-foi-anunciado-como-acesso-vitalicio_7zfD-D4s6GauY3fc/</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="12" t="inlineStr">
         <is>
-          <t>comprado. gostaria do reembolso assim que</t>
+          <t>plano freelancer imediato</t>
         </is>
       </c>
       <c r="B4" s="12" t="inlineStr">
         <is>
-          <t>comprado. Gostaria do reembolso assim que</t>
+          <t>Plano Freelancer Imediato</t>
         </is>
       </c>
       <c r="C4" s="12" t="inlineStr">
         <is>
-          <t>angulo</t>
+          <t>marca</t>
         </is>
       </c>
       <c r="D4" s="12" t="inlineStr">
@@ -953,74 +953,28 @@
       <c r="G4" s="12" t="n">
         <v>1</v>
       </c>
-      <c r="H4" s="12" t="inlineStr"/>
+      <c r="H4" s="12" t="inlineStr">
+        <is>
+          <t>R$ 11,00</t>
+        </is>
+      </c>
       <c r="I4" s="12" t="inlineStr">
         <is>
-          <t>2026-08-30</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="J4" s="12" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K4" s="12" t="inlineStr"/>
       <c r="L4" s="12" t="inlineStr">
         <is>
-          <t>https://www.reclameaqui.com.br/cakto-pay/pagamento-via-pix-nao-resultou-na-entrega-do-produto-solicitacao-de-reembolso-por-possivel-editado-pelo-reclame-aqui_cbUdm8Fq5-5oanwH/</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="12" t="inlineStr">
-        <is>
-          <t>curso online</t>
-        </is>
-      </c>
-      <c r="B5" s="12" t="inlineStr">
-        <is>
-          <t>curso online</t>
-        </is>
-      </c>
-      <c r="C5" s="12" t="inlineStr">
-        <is>
-          <t>angulo</t>
-        </is>
-      </c>
-      <c r="D5" s="12" t="inlineStr">
-        <is>
-          <t>Cakto</t>
-        </is>
-      </c>
-      <c r="E5" s="12" t="inlineStr">
-        <is>
-          <t>Ferramentas de IA / Produtividade</t>
-        </is>
-      </c>
-      <c r="F5" s="12" t="inlineStr">
-        <is>
-          <t>fria</t>
-        </is>
-      </c>
-      <c r="G5" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="H5" s="12" t="inlineStr"/>
-      <c r="I5" s="12" t="inlineStr">
-        <is>
-          <t>2026-08-30</t>
-        </is>
-      </c>
-      <c r="J5" s="12" t="n">
-        <v>3</v>
-      </c>
-      <c r="K5" s="12" t="inlineStr"/>
-      <c r="L5" s="12" t="inlineStr">
-        <is>
-          <t>https://www.reclameaqui.com.br/cakto-pay/curso-online-nao-entregue-apos-pagamento-com-falha-na-comunicacao-e-solicitacao-de-estorno_-bekag5hY78F-1mM/</t>
+          <t>https://www.reclameaqui.com.br/cakto-pay/plano-freelancer-imediato-pagamento-adicional-exigido-apos-compra-inicial-para-liberacao-de-acesso_Aa7b4b27tHVPApDH/</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L5"/>
+  <autoFilter ref="A1:L4"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1031,7 +985,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G3"/>
+  <dimension ref="A1:G4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -1087,10 +1041,10 @@
         </is>
       </c>
       <c r="B2" s="14" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C2" s="14" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D2" s="14" t="n">
         <v>0</v>
@@ -1102,23 +1056,23 @@
         <v>0</v>
       </c>
       <c r="G2" s="14" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="14" t="inlineStr">
         <is>
-          <t>Ferramentas de IA / Produtividade</t>
+          <t>Streaming e entretenimento</t>
         </is>
       </c>
       <c r="B3" s="14" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C3" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="D3" s="14" t="n">
         <v>0</v>
-      </c>
-      <c r="D3" s="14" t="n">
-        <v>2</v>
       </c>
       <c r="E3" s="14" t="n">
         <v>0</v>
@@ -1127,7 +1081,32 @@
         <v>0</v>
       </c>
       <c r="G3" s="14" t="n">
-        <v>2</v>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="14" t="inlineStr">
+        <is>
+          <t>Ferramentas de IA / Produtividade</t>
+        </is>
+      </c>
+      <c r="B4" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="C4" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="D4" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="E4" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="F4" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="G4" s="14" t="n">
+        <v>1</v>
       </c>
     </row>
   </sheetData>
@@ -1141,7 +1120,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C31"/>
+  <dimension ref="A1:C32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -1516,7 +1495,7 @@
         </is>
       </c>
       <c r="C22" s="14" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="23">
@@ -1546,7 +1525,7 @@
         </is>
       </c>
       <c r="C24" s="14" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="25">
@@ -1597,22 +1576,22 @@
     <row r="28">
       <c r="A28" s="14" t="inlineStr">
         <is>
-          <t>reembolso cakto dificuldade</t>
+          <t>plano freelancer imediato</t>
         </is>
       </c>
       <c r="B28" s="14" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="C28" s="14" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="14" t="inlineStr">
         <is>
-          <t>reembolso perfectpay recusa</t>
+          <t>reembolso cakto dificuldade</t>
         </is>
       </c>
       <c r="B29" s="14" t="inlineStr">
@@ -1627,31 +1606,46 @@
     <row r="30">
       <c r="A30" s="14" t="inlineStr">
         <is>
-          <t>spygram</t>
+          <t>reembolso perfectpay recusa</t>
         </is>
       </c>
       <c r="B30" s="14" t="inlineStr">
         <is>
-          <t>2026-08-30</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="C30" s="14" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="14" t="inlineStr">
         <is>
+          <t>spygram</t>
+        </is>
+      </c>
+      <c r="B31" s="14" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+      <c r="C31" s="14" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="14" t="inlineStr">
+        <is>
           <t>stalkeia</t>
         </is>
       </c>
-      <c r="B31" s="14" t="inlineStr">
+      <c r="B32" s="14" t="inlineStr">
         <is>
           <t>2026-08-30</t>
         </is>
       </c>
-      <c r="C31" s="14" t="n">
-        <v>2</v>
+      <c r="C32" s="14" t="n">
+        <v>3</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
radar 2026-09-01: +0 novas, 0 atualizadas, 0 snapshots
</commit_message>
<xml_diff>
--- a/Radar/radar-low-ticket.xlsx
+++ b/Radar/radar-low-ticket.xlsx
@@ -16,7 +16,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Resumo por nicho'!$A$1:$G$3</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Varredura'!$A$1:$D$7</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Achados'!$A$1:$L$11</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Achados'!$A$1:$L$6</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -736,7 +736,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L11"/>
+  <dimension ref="A1:L6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -818,17 +818,17 @@
     <row r="2">
       <c r="A2" s="12" t="inlineStr">
         <is>
-          <t>stalkeia</t>
+          <t>fica saindo e entrando sozinho</t>
         </is>
       </c>
       <c r="B2" s="12" t="inlineStr">
         <is>
-          <t>Stalkeia</t>
+          <t>fica saindo e entrando sozinho</t>
         </is>
       </c>
       <c r="C2" s="12" t="inlineStr">
         <is>
-          <t>marca</t>
+          <t>angulo</t>
         </is>
       </c>
       <c r="D2" s="12" t="inlineStr">
@@ -838,7 +838,7 @@
       </c>
       <c r="E2" s="12" t="inlineStr">
         <is>
-          <t>Espionagem e rastreamento</t>
+          <t>Ferramentas de IA / Produtividade</t>
         </is>
       </c>
       <c r="F2" s="12" t="inlineStr">
@@ -847,37 +847,33 @@
         </is>
       </c>
       <c r="G2" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="H2" s="12" t="inlineStr"/>
+      <c r="I2" s="12" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="J2" s="12" t="n">
         <v>2</v>
-      </c>
-      <c r="H2" s="12" t="inlineStr">
-        <is>
-          <t>R$ 47</t>
-        </is>
-      </c>
-      <c r="I2" s="12" t="inlineStr">
-        <is>
-          <t>2026-08-30</t>
-        </is>
-      </c>
-      <c r="J2" s="12" t="n">
-        <v>8</v>
       </c>
       <c r="K2" s="12" t="inlineStr"/>
       <c r="L2" s="12" t="inlineStr">
         <is>
-          <t>https://www.reclameaqui.com.br/perfectpay/propaganda-enganosa-do-e-solicitacao-de-reembolso-do-valor-pago_yID1cmkfVopy5OrZ/</t>
+          <t>https://www.reclameaqui.com.br/perfectpay/nao-gostei-do-app-fica-saindo-e-entrando-sozinho_UkdzKQ86egq0egAP/</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="12" t="inlineStr">
         <is>
-          <t>converza.io</t>
+          <t>método atlas</t>
         </is>
       </c>
       <c r="B3" s="12" t="inlineStr">
         <is>
-          <t>Converza.io</t>
+          <t>Método Atlas</t>
         </is>
       </c>
       <c r="C3" s="12" t="inlineStr">
@@ -887,12 +883,12 @@
       </c>
       <c r="D3" s="12" t="inlineStr">
         <is>
-          <t>Cakto</t>
+          <t>PerfectPay</t>
         </is>
       </c>
       <c r="E3" s="12" t="inlineStr">
         <is>
-          <t>Chatbots / Automação de mensagens</t>
+          <t>Educação e consultoria</t>
         </is>
       </c>
       <c r="F3" s="12" t="inlineStr">
@@ -912,37 +908,41 @@
       <c r="J3" s="12" t="n">
         <v>2</v>
       </c>
-      <c r="K3" s="12" t="inlineStr"/>
+      <c r="K3" s="12" t="inlineStr">
+        <is>
+          <t>Fiz uma compra desse tal método atlas, não cumpriu com prometido ,tento falar com suporte wattsap, e-mail e simplesmente desativaram as contas ,já procurei uma advogada e delegacia pra denunciar. Não caiam é [Editado pelo Reclame Aqui] RA Ads</t>
+        </is>
+      </c>
       <c r="L3" s="12" t="inlineStr">
         <is>
-          <t>https://www.reclameaqui.com.br/cakto-pay/exijo-reembolso-servico-nao-funciona-e-suporte-nao-responde_OPi-rimJXtkjo2yB/</t>
+          <t>https://www.reclameaqui.com.br/perfectpay/compra-do-metodo-atlas-nao-cumpre-o-prometido-e-suporte-desativado_wzci0DCEtGCFBRc6/</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="12" t="inlineStr">
         <is>
-          <t>comunidade vsa</t>
+          <t>interactive live</t>
         </is>
       </c>
       <c r="B4" s="12" t="inlineStr">
         <is>
-          <t>COMUNIDADE VSA</t>
+          <t>Interactive Live</t>
         </is>
       </c>
       <c r="C4" s="12" t="inlineStr">
         <is>
-          <t>marca</t>
+          <t>angulo</t>
         </is>
       </c>
       <c r="D4" s="12" t="inlineStr">
         <is>
-          <t>Cakto</t>
+          <t>PerfectPay</t>
         </is>
       </c>
       <c r="E4" s="12" t="inlineStr">
         <is>
-          <t>Marketing / Comunidades de negócios</t>
+          <t>Espionagem e rastreamento</t>
         </is>
       </c>
       <c r="F4" s="12" t="inlineStr">
@@ -953,11 +953,7 @@
       <c r="G4" s="12" t="n">
         <v>1</v>
       </c>
-      <c r="H4" s="12" t="inlineStr">
-        <is>
-          <t>R$ 248,89.</t>
-        </is>
-      </c>
+      <c r="H4" s="12" t="inlineStr"/>
       <c r="I4" s="12" t="inlineStr">
         <is>
           <t>2026-08-31</t>
@@ -966,27 +962,31 @@
       <c r="J4" s="12" t="n">
         <v>2</v>
       </c>
-      <c r="K4" s="12" t="inlineStr"/>
+      <c r="K4" s="12" t="inlineStr">
+        <is>
+          <t>Comprei o produto "Interactive Live" através da plataforma Perfect Pay, que atuou como processadora de pagamento da venda. O produto recebido não correspondeu ao que foi anunciado/esperado, e eu solicitei o cancelamento/reembolso ainda dentro do prazo de garantia de 7 dias previsto no site/checkout, que também é assegurado pelo direito de arrependimento do art. 49 do Código de Defesa do Consumidor para compras feitas fora do estabelecimento comercial (como é o caso de compras online). Esse prazo</t>
+        </is>
+      </c>
       <c r="L4" s="12" t="inlineStr">
         <is>
-          <t>https://www.reclameaqui.com.br/cakto-pay/solicitacao-de-reembolso-de-compra-com-erro-de-saldo-na-conta-do-vendedor_e5d-tH3gUGahNktM/</t>
+          <t>https://www.reclameaqui.com.br/perfectpay/reembolso-negado-e-prazo-expirado-devido-a-burocracia-da-perfect-pay_wFj48yi7DgllZO-Z/</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="12" t="inlineStr">
         <is>
-          <t>retrato da sua alma gêmea</t>
+          <t>low ticket do zero 2.0 no dia 30</t>
         </is>
       </c>
       <c r="B5" s="12" t="inlineStr">
         <is>
-          <t>Retrato da Sua Alma Gêmea</t>
+          <t>Low Ticket do Zero 2.0 no dia 30</t>
         </is>
       </c>
       <c r="C5" s="12" t="inlineStr">
         <is>
-          <t>marca</t>
+          <t>angulo</t>
         </is>
       </c>
       <c r="D5" s="12" t="inlineStr">
@@ -996,7 +996,7 @@
       </c>
       <c r="E5" s="12" t="inlineStr">
         <is>
-          <t>Arte personalizada / IA generativa</t>
+          <t>Ferramentas de IA / Produtividade</t>
         </is>
       </c>
       <c r="F5" s="12" t="inlineStr">
@@ -1007,11 +1007,7 @@
       <c r="G5" s="12" t="n">
         <v>1</v>
       </c>
-      <c r="H5" s="12" t="inlineStr">
-        <is>
-          <t>R$ 48,89</t>
-        </is>
-      </c>
+      <c r="H5" s="12" t="inlineStr"/>
       <c r="I5" s="12" t="inlineStr">
         <is>
           <t>2026-08-31</t>
@@ -1020,27 +1016,31 @@
       <c r="J5" s="12" t="n">
         <v>2</v>
       </c>
-      <c r="K5" s="12" t="inlineStr"/>
+      <c r="K5" s="12" t="inlineStr">
+        <is>
+          <t>Solicitação de cancelamento e reembolso negada por falta de saldo na conta do produtor. Resolvido CAKTO PAY Rio de Janeiro - RJ 31/08/2026 às 17:20</t>
+        </is>
+      </c>
       <c r="L5" s="12" t="inlineStr">
         <is>
-          <t>https://www.reclameaqui.com.br/cakto-pay/editado-pelo-reclame-aqui-e-solicitacao-de-estorno-para-produto-retrato-da-sua-alma-gemea_H8ihRLGIEQMZ9WSb/</t>
+          <t>https://www.reclameaqui.com.br/cakto-pay/solicitacao-de-cancelamento-e-reembolso-negada-por-falta-de-saldo-na-conta-do-produtor_g_uRVUXcpBO7YtT5/</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="12" t="inlineStr">
         <is>
-          <t>pack canva happy hour</t>
+          <t>um aplicativo</t>
         </is>
       </c>
       <c r="B6" s="12" t="inlineStr">
         <is>
-          <t>Pack Canva Happy Hour</t>
+          <t>um aplicativo</t>
         </is>
       </c>
       <c r="C6" s="12" t="inlineStr">
         <is>
-          <t>marca</t>
+          <t>angulo</t>
         </is>
       </c>
       <c r="D6" s="12" t="inlineStr">
@@ -1050,7 +1050,7 @@
       </c>
       <c r="E6" s="12" t="inlineStr">
         <is>
-          <t>PLR / Produtos digitais para revenda</t>
+          <t>Infoprodutos - suporte e reembolso</t>
         </is>
       </c>
       <c r="F6" s="12" t="inlineStr">
@@ -1061,11 +1061,7 @@
       <c r="G6" s="12" t="n">
         <v>1</v>
       </c>
-      <c r="H6" s="12" t="inlineStr">
-        <is>
-          <t>R$ 15,15</t>
-        </is>
-      </c>
+      <c r="H6" s="12" t="inlineStr"/>
       <c r="I6" s="12" t="inlineStr">
         <is>
           <t>2026-08-31</t>
@@ -1074,281 +1070,19 @@
       <c r="J6" s="12" t="n">
         <v>2</v>
       </c>
-      <c r="K6" s="12" t="inlineStr"/>
+      <c r="K6" s="12" t="inlineStr">
+        <is>
+          <t>Fiz uma compra de um aplicativo, porém o mesmo não funciona, entrei em contato com a cakto por email, entrei em contato pelo suporte da plataforma e não me respondem, foi uma compra de +- 840 reais Quero o reembolso da minha compra: Dados da compra: Poxa, vou te ajudar a resolver isso! Me informe: Qual e-mail você usou na compra?</t>
+        </is>
+      </c>
       <c r="L6" s="12" t="inlineStr">
         <is>
-          <t>https://www.reclameaqui.com.br/cakto-pay/solicitacao-de-cancelamento-e-reembolso-de-cursos-online-apos-arrependimento-de-compra_-CZPnDHntp_r19_O/</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="12" t="inlineStr">
-        <is>
-          <t>fica saindo e entrando sozinho</t>
-        </is>
-      </c>
-      <c r="B7" s="12" t="inlineStr">
-        <is>
-          <t>fica saindo e entrando sozinho</t>
-        </is>
-      </c>
-      <c r="C7" s="12" t="inlineStr">
-        <is>
-          <t>angulo</t>
-        </is>
-      </c>
-      <c r="D7" s="12" t="inlineStr">
-        <is>
-          <t>PerfectPay</t>
-        </is>
-      </c>
-      <c r="E7" s="12" t="inlineStr">
-        <is>
-          <t>Ferramentas de IA / Produtividade</t>
-        </is>
-      </c>
-      <c r="F7" s="12" t="inlineStr">
-        <is>
-          <t>fria</t>
-        </is>
-      </c>
-      <c r="G7" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="H7" s="12" t="inlineStr"/>
-      <c r="I7" s="12" t="inlineStr">
-        <is>
-          <t>2026-08-31</t>
-        </is>
-      </c>
-      <c r="J7" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="K7" s="12" t="inlineStr"/>
-      <c r="L7" s="12" t="inlineStr">
-        <is>
-          <t>https://www.reclameaqui.com.br/perfectpay/nao-gostei-do-app-fica-saindo-e-entrando-sozinho_UkdzKQ86egq0egAP/</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="12" t="inlineStr">
-        <is>
-          <t>método atlas</t>
-        </is>
-      </c>
-      <c r="B8" s="12" t="inlineStr">
-        <is>
-          <t>Método Atlas</t>
-        </is>
-      </c>
-      <c r="C8" s="12" t="inlineStr">
-        <is>
-          <t>marca</t>
-        </is>
-      </c>
-      <c r="D8" s="12" t="inlineStr">
-        <is>
-          <t>PerfectPay</t>
-        </is>
-      </c>
-      <c r="E8" s="12" t="inlineStr">
-        <is>
-          <t>Educação e consultoria</t>
-        </is>
-      </c>
-      <c r="F8" s="12" t="inlineStr">
-        <is>
-          <t>fria</t>
-        </is>
-      </c>
-      <c r="G8" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="H8" s="12" t="inlineStr"/>
-      <c r="I8" s="12" t="inlineStr">
-        <is>
-          <t>2026-08-31</t>
-        </is>
-      </c>
-      <c r="J8" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="K8" s="12" t="inlineStr">
-        <is>
-          <t>Fiz uma compra desse tal método atlas, não cumpriu com prometido ,tento falar com suporte wattsap, e-mail e simplesmente desativaram as contas ,já procurei uma advogada e delegacia pra denunciar. Não caiam é [Editado pelo Reclame Aqui] RA Ads</t>
-        </is>
-      </c>
-      <c r="L8" s="12" t="inlineStr">
-        <is>
-          <t>https://www.reclameaqui.com.br/perfectpay/compra-do-metodo-atlas-nao-cumpre-o-prometido-e-suporte-desativado_wzci0DCEtGCFBRc6/</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="12" t="inlineStr">
-        <is>
-          <t>interactive live</t>
-        </is>
-      </c>
-      <c r="B9" s="12" t="inlineStr">
-        <is>
-          <t>Interactive Live</t>
-        </is>
-      </c>
-      <c r="C9" s="12" t="inlineStr">
-        <is>
-          <t>angulo</t>
-        </is>
-      </c>
-      <c r="D9" s="12" t="inlineStr">
-        <is>
-          <t>PerfectPay</t>
-        </is>
-      </c>
-      <c r="E9" s="12" t="inlineStr">
-        <is>
-          <t>Espionagem e rastreamento</t>
-        </is>
-      </c>
-      <c r="F9" s="12" t="inlineStr">
-        <is>
-          <t>fria</t>
-        </is>
-      </c>
-      <c r="G9" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="H9" s="12" t="inlineStr"/>
-      <c r="I9" s="12" t="inlineStr">
-        <is>
-          <t>2026-08-31</t>
-        </is>
-      </c>
-      <c r="J9" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="K9" s="12" t="inlineStr">
-        <is>
-          <t>Comprei o produto "Interactive Live" através da plataforma Perfect Pay, que atuou como processadora de pagamento da venda. O produto recebido não correspondeu ao que foi anunciado/esperado, e eu solicitei o cancelamento/reembolso ainda dentro do prazo de garantia de 7 dias previsto no site/checkout, que também é assegurado pelo direito de arrependimento do art. 49 do Código de Defesa do Consumidor para compras feitas fora do estabelecimento comercial (como é o caso de compras online). Esse prazo</t>
-        </is>
-      </c>
-      <c r="L9" s="12" t="inlineStr">
-        <is>
-          <t>https://www.reclameaqui.com.br/perfectpay/reembolso-negado-e-prazo-expirado-devido-a-burocracia-da-perfect-pay_wFj48yi7DgllZO-Z/</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="12" t="inlineStr">
-        <is>
-          <t>low ticket do zero 2.0 no dia 30</t>
-        </is>
-      </c>
-      <c r="B10" s="12" t="inlineStr">
-        <is>
-          <t>Low Ticket do Zero 2.0 no dia 30</t>
-        </is>
-      </c>
-      <c r="C10" s="12" t="inlineStr">
-        <is>
-          <t>angulo</t>
-        </is>
-      </c>
-      <c r="D10" s="12" t="inlineStr">
-        <is>
-          <t>Cakto</t>
-        </is>
-      </c>
-      <c r="E10" s="12" t="inlineStr">
-        <is>
-          <t>Ferramentas de IA / Produtividade</t>
-        </is>
-      </c>
-      <c r="F10" s="12" t="inlineStr">
-        <is>
-          <t>fria</t>
-        </is>
-      </c>
-      <c r="G10" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="H10" s="12" t="inlineStr"/>
-      <c r="I10" s="12" t="inlineStr">
-        <is>
-          <t>2026-08-31</t>
-        </is>
-      </c>
-      <c r="J10" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="K10" s="12" t="inlineStr">
-        <is>
-          <t>Solicitação de cancelamento e reembolso negada por falta de saldo na conta do produtor. Não respondida CAKTO PAY Rio de Janeiro - RJ 31/08/2026 às 17:20</t>
-        </is>
-      </c>
-      <c r="L10" s="12" t="inlineStr">
-        <is>
-          <t>https://www.reclameaqui.com.br/cakto-pay/solicitacao-de-cancelamento-e-reembolso-negada-por-falta-de-saldo-na-conta-do-produtor_g_uRVUXcpBO7YtT5/</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="12" t="inlineStr">
-        <is>
-          <t>um aplicativo</t>
-        </is>
-      </c>
-      <c r="B11" s="12" t="inlineStr">
-        <is>
-          <t>um aplicativo</t>
-        </is>
-      </c>
-      <c r="C11" s="12" t="inlineStr">
-        <is>
-          <t>angulo</t>
-        </is>
-      </c>
-      <c r="D11" s="12" t="inlineStr">
-        <is>
-          <t>Cakto</t>
-        </is>
-      </c>
-      <c r="E11" s="12" t="inlineStr">
-        <is>
-          <t>Infoprodutos - suporte e reembolso</t>
-        </is>
-      </c>
-      <c r="F11" s="12" t="inlineStr">
-        <is>
-          <t>fria</t>
-        </is>
-      </c>
-      <c r="G11" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="H11" s="12" t="inlineStr"/>
-      <c r="I11" s="12" t="inlineStr">
-        <is>
-          <t>2026-08-31</t>
-        </is>
-      </c>
-      <c r="J11" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="K11" s="12" t="inlineStr">
-        <is>
-          <t>Fiz uma compra de um aplicativo, porém o mesmo não funciona, entrei em contato com a cakto por email, entrei em contato pelo suporte da plataforma e não me respondem, foi uma compra de +- 840 reais Quero o reembolso da minha compra: Dados da compra: Poxa, vou te ajudar a resolver isso! Me informe: Qual e-mail você usou na compra?</t>
-        </is>
-      </c>
-      <c r="L11" s="12" t="inlineStr">
-        <is>
           <t>https://www.reclameaqui.com.br/cakto-pay/reclamacao-sobre-aplicativo-nao-funcional-e-falta-de-resposta-do-suporte-para-reembolso_vE-W5K4jwJY0jtXa/</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L11"/>
+  <autoFilter ref="A1:L6"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1359,7 +1093,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G9"/>
+  <dimension ref="A1:G5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -1411,17 +1145,17 @@
     <row r="2">
       <c r="A2" s="14" t="inlineStr">
         <is>
-          <t>Espionagem e rastreamento</t>
+          <t>Ferramentas de IA / Produtividade</t>
         </is>
       </c>
       <c r="B2" s="14" t="n">
         <v>2</v>
       </c>
       <c r="C2" s="14" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D2" s="14" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E2" s="14" t="n">
         <v>0</v>
@@ -1436,17 +1170,17 @@
     <row r="3">
       <c r="A3" s="14" t="inlineStr">
         <is>
-          <t>Ferramentas de IA / Produtividade</t>
+          <t>Educação e consultoria</t>
         </is>
       </c>
       <c r="B3" s="14" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C3" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="D3" s="14" t="n">
         <v>0</v>
-      </c>
-      <c r="D3" s="14" t="n">
-        <v>2</v>
       </c>
       <c r="E3" s="14" t="n">
         <v>0</v>
@@ -1455,23 +1189,23 @@
         <v>0</v>
       </c>
       <c r="G3" s="14" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="14" t="inlineStr">
         <is>
-          <t>Chatbots / Automação de mensagens</t>
+          <t>Espionagem e rastreamento</t>
         </is>
       </c>
       <c r="B4" s="14" t="n">
         <v>1</v>
       </c>
       <c r="C4" s="14" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D4" s="14" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E4" s="14" t="n">
         <v>0</v>
@@ -1486,17 +1220,17 @@
     <row r="5">
       <c r="A5" s="14" t="inlineStr">
         <is>
-          <t>Marketing / Comunidades de negócios</t>
+          <t>Infoprodutos - suporte e reembolso</t>
         </is>
       </c>
       <c r="B5" s="14" t="n">
         <v>1</v>
       </c>
       <c r="C5" s="14" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D5" s="14" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E5" s="14" t="n">
         <v>0</v>
@@ -1505,106 +1239,6 @@
         <v>0</v>
       </c>
       <c r="G5" s="14" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="14" t="inlineStr">
-        <is>
-          <t>Arte personalizada / IA generativa</t>
-        </is>
-      </c>
-      <c r="B6" s="14" t="n">
-        <v>1</v>
-      </c>
-      <c r="C6" s="14" t="n">
-        <v>1</v>
-      </c>
-      <c r="D6" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="E6" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="F6" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="G6" s="14" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="14" t="inlineStr">
-        <is>
-          <t>PLR / Produtos digitais para revenda</t>
-        </is>
-      </c>
-      <c r="B7" s="14" t="n">
-        <v>1</v>
-      </c>
-      <c r="C7" s="14" t="n">
-        <v>1</v>
-      </c>
-      <c r="D7" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="E7" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="F7" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="G7" s="14" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="14" t="inlineStr">
-        <is>
-          <t>Educação e consultoria</t>
-        </is>
-      </c>
-      <c r="B8" s="14" t="n">
-        <v>1</v>
-      </c>
-      <c r="C8" s="14" t="n">
-        <v>1</v>
-      </c>
-      <c r="D8" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="E8" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="F8" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="G8" s="14" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="14" t="inlineStr">
-        <is>
-          <t>Infoprodutos - suporte e reembolso</t>
-        </is>
-      </c>
-      <c r="B9" s="14" t="n">
-        <v>1</v>
-      </c>
-      <c r="C9" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="D9" s="14" t="n">
-        <v>1</v>
-      </c>
-      <c r="E9" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="F9" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="G9" s="14" t="n">
         <v>1</v>
       </c>
     </row>
@@ -2009,7 +1643,7 @@
         </is>
       </c>
       <c r="C23" s="14" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="24">
@@ -2039,7 +1673,7 @@
         </is>
       </c>
       <c r="C25" s="14" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="26">
@@ -2084,7 +1718,7 @@
         </is>
       </c>
       <c r="C28" s="14" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="29">
@@ -2144,7 +1778,7 @@
         </is>
       </c>
       <c r="C32" s="14" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="33">
@@ -2159,7 +1793,7 @@
         </is>
       </c>
       <c r="C33" s="14" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="34">
@@ -2204,7 +1838,7 @@
         </is>
       </c>
       <c r="C36" s="14" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="37">
@@ -2219,7 +1853,7 @@
         </is>
       </c>
       <c r="C37" s="14" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="38">
@@ -2294,7 +1928,7 @@
         </is>
       </c>
       <c r="C42" s="14" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="43">
@@ -2324,7 +1958,7 @@
         </is>
       </c>
       <c r="C44" s="14" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="45">
@@ -2339,7 +1973,7 @@
         </is>
       </c>
       <c r="C45" s="14" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="46">

</xml_diff>

<commit_message>
radar 2026-09-02: +0 novas, 0 atualizadas, 0 snapshots
</commit_message>
<xml_diff>
--- a/Radar/radar-low-ticket.xlsx
+++ b/Radar/radar-low-ticket.xlsx
@@ -12,7 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Historico" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Achados'!$A$1:$L$12</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Achados'!$A$1:$L$28</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -441,7 +441,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L12"/>
+  <dimension ref="A1:L28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -523,27 +523,27 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>stalkeia</t>
+          <t>fábrica de low ticket</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Stalkeia</t>
+          <t>Fábrica de Low Ticket</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>marca</t>
+          <t>angulo</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>PerfectPay</t>
+          <t>Cakto</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Espionagem e rastreamento</t>
+          <t>Educação / Marketing digital e low ticket</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
@@ -552,11 +552,11 @@
         </is>
       </c>
       <c r="G2" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>R$ 47</t>
+          <t>R$ 254,98</t>
         </is>
       </c>
       <c r="I2" s="2" t="inlineStr">
@@ -565,33 +565,33 @@
         </is>
       </c>
       <c r="J2" s="2" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="K2" s="2" t="inlineStr">
         <is>
-          <t>RA Ads Veja também todas as reclamações não respondidas respondidas finalizadas propaganda enganosa do Stalkeia.app e solicitação de reembolso do valor pago.  Resolvido  PerfectPay  Goiânia - GO  31/08/2026 às 04:47  ID: 257782105  realizei o pagamento direto no aplicativo, que prometia te entregar</t>
+          <t>Adquiri o curso com base na promessa apresentada pelo produtor de que haveria suporte individual. Porém, após entrar no grupo de WhatsApp, me deparei com uma discussão entre outros alunos que estavam reclamando justamente sobre essa questão. Na conversa, um dos administradores informou que a estratégia havia sido alterada e que o suporte agora seria realizado de forma coletiva pelo grupo. Eu não fui comunicado previamente sobre essa mudança e essa não foi a condição pela qual adquiri o curso. Co</t>
         </is>
       </c>
       <c r="L2" s="2" t="inlineStr">
         <is>
-          <t>https://www.reclameaqui.com.br/perfectpay/propaganda-enganosa-do-e-solicitacao-de-reembolso-do-valor-pago_yID1cmkfVopy5OrZ/</t>
+          <t>https://www.reclameaqui.com.br/cakto-pay/reembolso-solicitado-por-propaganda-enganosa-sobre-suporte-individual-no-curso-fabrica-de-low-ticket_BQx79JwlEi7-NBzU/</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>fábrica de low ticket</t>
+          <t>on line rj comercio varejista de acessorios ltda</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Fábrica de Low Ticket</t>
+          <t>On Line Rj Comercio Varejista De Acessorios Ltda</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>marca</t>
+          <t>angulo</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
@@ -601,7 +601,7 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>Ganhar dinheiro online / trabalho remoto</t>
+          <t>Espionagem e rastreamento</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
@@ -614,7 +614,7 @@
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>R$ 254,98</t>
+          <t>R$ 297,00</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
@@ -623,28 +623,24 @@
         </is>
       </c>
       <c r="J3" s="2" t="n">
-        <v>7</v>
-      </c>
-      <c r="K3" s="2" t="inlineStr">
-        <is>
-          <t>Veja também todas as reclamações não respondidas respondidas finalizadas Reembolso solicitado por propaganda enganosa sobre suporte individual no curso Fábrica de Low Ticket  Resolvido  CAKTO PAY  Cansanção - BA  01/09/2026 às 08:18  ID: 257896487  Olá,  Solicito o reembolso da compra da Fábrica de</t>
-        </is>
-      </c>
+        <v>4</v>
+      </c>
+      <c r="K3" s="2" t="inlineStr"/>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>https://www.reclameaqui.com.br/cakto-pay/reembolso-solicitado-por-propaganda-enganosa-sobre-suporte-individual-no-curso-fabrica-de-low-ticket_BQx79JwlEi7-NBzU/</t>
+          <t>https://www.reclameaqui.com.br/cakto-pay/solicitacao-de-reembolso-de-assinatura-tokfy-via-pix-devido-a-plano-incorreto-e-falha-no-login-para-cancelamento_lwKWxoGQVq5QbJLn/</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>um curso e</t>
+          <t>fica saindo e entrando sozinho</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>um curso e</t>
+          <t>fica saindo e entrando sozinho</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
@@ -659,7 +655,7 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Educação e consultoria</t>
+          <t>Ferramentas de IA / Produtividade</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
@@ -673,37 +669,33 @@
       <c r="H4" s="2" t="inlineStr"/>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="J4" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="K4" s="2" t="inlineStr">
-        <is>
-          <t>RA Ads Veja também todas as reclamações não respondidas respondidas finalizadas [Editado pelo Reclame Aqui]  Resolvido  PerfectPay  Osasco - SP  31/08/2026 às 00:24  ID: 257779321  Fiz compra de um curso e é [Editado pelo Reclame Aqui]. Quero [Editado pelo Reclame Aqui] código *****  Aguardo.  RA Ad</t>
-        </is>
-      </c>
+        <v>6</v>
+      </c>
+      <c r="K4" s="2" t="inlineStr"/>
       <c r="L4" s="2" t="inlineStr">
         <is>
-          <t>https://www.reclameaqui.com.br/perfectpay/editado-pelo-reclame-aqui_UeZdzzFsRKKhakiR/</t>
+          <t>https://www.reclameaqui.com.br/perfectpay/nao-gostei-do-app-fica-saindo-e-entrando-sozinho_UkdzKQ86egq0egAP/</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>ra ads previous slide next slide compartilhe resp</t>
+          <t>método atlas</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>RA Ads Previous slide Next slide Compartilhe Resp</t>
+          <t>Método Atlas</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>angulo</t>
+          <t>marca</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
@@ -713,7 +705,7 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Ferramentas de IA / Produtividade</t>
+          <t>Educação e consultoria</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
@@ -727,32 +719,32 @@
       <c r="H5" s="2" t="inlineStr"/>
       <c r="I5" s="2" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="J5" s="2" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="K5" s="2" t="inlineStr">
         <is>
-          <t>RA Ads Veja também todas as reclamações não respondidas respondidas finalizadas [Editado pelo Reclame Aqui]  Resolvido  PerfectPay  Mogi das Cruzes - SP  30/08/2026 às 23:05  ID: 257777077  Sofia um [Editado pelo Reclame Aqui], paguei e não recebi o produto  RA Ads Previous slide Next slide  Compart</t>
+          <t>Fiz uma compra desse tal método atlas, não cumpriu com prometido ,tento falar com suporte wattsap, e-mail e simplesmente desativaram as contas ,já procurei uma advogada e delegacia pra denunciar. Não caiam é [Editado pelo Reclame Aqui] RA Ads</t>
         </is>
       </c>
       <c r="L5" s="2" t="inlineStr">
         <is>
-          <t>https://www.reclameaqui.com.br/perfectpay/editado-pelo-reclame-aqui_SUXSgNqlxlTtM8rF/</t>
+          <t>https://www.reclameaqui.com.br/perfectpay/compra-do-metodo-atlas-nao-cumpre-o-prometido-e-suporte-desativado_wzci0DCEtGCFBRc6/</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>e ele nao chegou quero meu dinheiro de volta ra ad</t>
+          <t>interactive live</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>e ele nao chegou quero meu dinheiro de volta RA Ad</t>
+          <t>Interactive Live</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
@@ -767,7 +759,7 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Ferramentas de IA / Produtividade</t>
+          <t>Espionagem e rastreamento</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
@@ -781,37 +773,37 @@
       <c r="H6" s="2" t="inlineStr"/>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="J6" s="2" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="K6" s="2" t="inlineStr">
         <is>
-          <t>RA Ads Veja também todas as reclamações não respondidas respondidas finalizadas Propaganda inganosa  Respondida  PerfectPay  Caxias do Sul - RS  30/08/2026 às 15:07  ID: 257755023     Fiz a compra de um produto e ele nao chegou quero meu dinheiro de volta  RA Ads Previous slide Next slide  Compartil</t>
+          <t>Comprei o produto "Interactive Live" através da plataforma Perfect Pay, que atuou como processadora de pagamento da venda. O produto recebido não correspondeu ao que foi anunciado/esperado, e eu solicitei o cancelamento/reembolso ainda dentro do prazo de garantia de 7 dias previsto no site/checkout, que também é assegurado pelo direito de arrependimento do art. 49 do Código de Defesa do Consumidor para compras feitas fora do estabelecimento comercial (como é o caso de compras online). Esse prazo</t>
         </is>
       </c>
       <c r="L6" s="2" t="inlineStr">
         <is>
-          <t>https://www.reclameaqui.com.br/perfectpay/propaganda-inganosa_WXGZ3QLZ1OhfoBjb/</t>
+          <t>https://www.reclameaqui.com.br/perfectpay/reembolso-negado-e-prazo-expirado-devido-a-burocracia-da-perfect-pay_wFj48yi7DgllZO-Z/</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>converza.io</t>
+          <t>low ticket do zero 2.0 no dia 30</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Converza.io</t>
+          <t>Low Ticket do Zero 2.0 no dia 30</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>marca</t>
+          <t>angulo</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
@@ -835,37 +827,37 @@
       <c r="H7" s="2" t="inlineStr"/>
       <c r="I7" s="2" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="J7" s="2" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="K7" s="2" t="inlineStr">
         <is>
-          <t>RA Ads Veja também todas as reclamações não respondidas respondidas finalizadas Exijo reembolso serviço não funciona e suporte não responde  Respondida  CAKTO PAY  São Paulo - SP  31/08/2026 às 03:25  ID: 257781633  Assinei um plano da Converza.io, porém não consigo sequer criar um dispositivo para</t>
+          <t>Solicitação de cancelamento e reembolso negada por falta de saldo na conta do produtor. Resolvido CAKTO PAY Rio de Janeiro - RJ 31/08/2026 às 17:20</t>
         </is>
       </c>
       <c r="L7" s="2" t="inlineStr">
         <is>
-          <t>https://www.reclameaqui.com.br/cakto-pay/exijo-reembolso-servico-nao-funciona-e-suporte-nao-responde_OPi-rimJXtkjo2yB/</t>
+          <t>https://www.reclameaqui.com.br/cakto-pay/solicitacao-de-cancelamento-e-reembolso-negada-por-falta-de-saldo-na-conta-do-produtor_g_uRVUXcpBO7YtT5/</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>comunidade vsa</t>
+          <t>cloakeuai</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>COMUNIDADE VSA</t>
+          <t>Cloakeuai</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>marca</t>
+          <t>angulo</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
@@ -875,7 +867,7 @@
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>Espionagem e rastreamento</t>
+          <t>Ferramentas de IA / Cloaking</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
@@ -886,54 +878,50 @@
       <c r="G8" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="H8" s="2" t="inlineStr">
-        <is>
-          <t>R$ 248,89.</t>
-        </is>
-      </c>
+      <c r="H8" s="2" t="inlineStr"/>
       <c r="I8" s="2" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="J8" s="2" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="K8" s="2" t="inlineStr">
         <is>
-          <t>RA Ads Veja também todas as reclamações não respondidas respondidas finalizadas Solicitação de reembolso de compra com erro de saldo na conta do vendedor  Respondida  CAKTO PAY  Junqueiro - AL  31/08/2026 às 02:34  ID: 257781211  Olá,  Solicito o reembolso da compra da COMUNIDADE VSA, realizada em 2</t>
+          <t>Fiz uma compra de um aplicativo, porém o mesmo não funciona, entrei em contato com a cakto por email, entrei em contato pelo suporte da plataforma e não me respondem, foi uma compra de +- 840 reais Quero o reembolso da minha compra: Dados da compra: Poxa, vou te ajudar a resolver isso! Me informe: Qual e-mail você usou na compra?</t>
         </is>
       </c>
       <c r="L8" s="2" t="inlineStr">
         <is>
-          <t>https://www.reclameaqui.com.br/cakto-pay/solicitacao-de-reembolso-de-compra-com-erro-de-saldo-na-conta-do-vendedor_e5d-tH3gUGahNktM/</t>
+          <t>https://www.reclameaqui.com.br/cakto-pay/reclamacao-sobre-aplicativo-nao-funcional-e-falta-de-resposta-do-suporte-para-reembolso_vE-W5K4jwJY0jtXa/</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>retrato da sua alma gêmea</t>
+          <t>códigos lucrativos</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Retrato da Sua Alma Gêmea</t>
+          <t>Códigos Lucrativos</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>marca</t>
+          <t>angulo</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>Cakto</t>
+          <t>PerfectPay</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>Ferramentas de IA / Produtividade</t>
+          <t>Ganhar dinheiro online / Ferramentas de afiliado</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
@@ -944,54 +932,50 @@
       <c r="G9" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="H9" s="2" t="inlineStr">
-        <is>
-          <t>R$ 48,89</t>
-        </is>
-      </c>
+      <c r="H9" s="2" t="inlineStr"/>
       <c r="I9" s="2" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="J9" s="2" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="K9" s="2" t="inlineStr">
         <is>
-          <t>RA Ads Veja também todas as reclamações não respondidas respondidas finalizadas [Editado pelo Reclame Aqui] e solicitação de estorno para produto "Retrato da Sua Alma Gêmea"  Respondida  CAKTO PAY  Campinas - SP  31/08/2026 às 02:06  ID: 257780917  Olá, equipe da Cakto Pay,No dia 28/08/2026, realize</t>
+          <t>Comprei dois aplicativos codigos lucrativos e opinipix pela perfect pay,mas eles são [Editado pelo Reclame Aqui] . [Editado pelo Reclame Aqui]. Quero meu dinheiro de volta. Resposta da Empresa 31/01/2025 às 17:31</t>
         </is>
       </c>
       <c r="L9" s="2" t="inlineStr">
         <is>
-          <t>https://www.reclameaqui.com.br/cakto-pay/editado-pelo-reclame-aqui-e-solicitacao-de-estorno-para-produto-retrato-da-sua-alma-gemea_H8ihRLGIEQMZ9WSb/</t>
+          <t>https://www.reclameaqui.com.br/perfectpay/compra-de-aplicativos-editado-pelo-reclame-aqui-e-editado-pelo-reclame-aqui-solicitacao-de-reembolso_xx2YJjct0gsb0fGa/</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>pack canva</t>
+          <t>aristocracy negócios digitais</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Pack Canva</t>
+          <t>Aristocracy Negócios Digitais</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>marca</t>
+          <t>angulo</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>Cakto</t>
+          <t>PerfectPay</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>Educação e consultoria</t>
+          <t>Produtos digitais variados / Assinatura vitalícia</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
@@ -1002,27 +986,19 @@
       <c r="G10" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="H10" s="2" t="inlineStr">
-        <is>
-          <t>R$ 15,15</t>
-        </is>
-      </c>
+      <c r="H10" s="2" t="inlineStr"/>
       <c r="I10" s="2" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="J10" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="K10" s="2" t="inlineStr">
-        <is>
-          <t>RA Ads Veja também todas as reclamações não respondidas respondidas finalizadas Solicitação de cancelamento e reembolso de cursos online após arrependimento de compra.  Respondida  CAKTO PAY  Suzano - SP  30/08/2026 às 19:54  ID: 257768163  Me chamo *****, solicito o cancelamento e reembolso do valo</t>
-        </is>
-      </c>
+        <v>6</v>
+      </c>
+      <c r="K10" s="2" t="inlineStr"/>
       <c r="L10" s="2" t="inlineStr">
         <is>
-          <t>https://www.reclameaqui.com.br/cakto-pay/solicitacao-de-cancelamento-e-reembolso-de-cursos-online-apos-arrependimento-de-compra_-CZPnDHntp_r19_O/</t>
+          <t>https://www.reclameaqui.com.br/perfectpay/acesso-negado-a-produtos-com-assinatura-vitalicia-e-namorada-customizada-nao-funciona_VUCzPEy-WEHTKJWB/</t>
         </is>
       </c>
     </row>
@@ -1039,7 +1015,7 @@
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>marca</t>
+          <t>angulo</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
@@ -1049,7 +1025,7 @@
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>Espionagem e rastreamento</t>
+          <t>Ferramentas de espionagem / WhatsApp</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
@@ -1067,11 +1043,11 @@
         </is>
       </c>
       <c r="J11" s="2" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="K11" s="2" t="inlineStr">
         <is>
-          <t>Veja também todas as reclamações não respondidas respondidas finalizadas Solicitação de estorno de compra no site ZAP Radar por não recebimento de relatório.  Respondida  PerfectPay  Niterói - RJ  31/08/2026 às 22:22  ID: 257882275  Fiz uma compra no valor de 137,00 site ZAP radar e fui [Editado pel</t>
+          <t>Fiz uma compra no valor de 137,00 site ZAP radar e fui [Editado pelo Reclame Aqui] porque não abre um relatório. Peço o estorno do valor pago. RA Ads</t>
         </is>
       </c>
       <c r="L11" s="2" t="inlineStr">
@@ -1083,7 +1059,7 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>apostila de psicologia025</t>
+          <t>apostila de psicologia 2025</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
@@ -1093,7 +1069,7 @@
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>marca</t>
+          <t>angulo</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
@@ -1103,7 +1079,7 @@
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>Educação e consultoria</t>
+          <t>Educação / Concursos e certificações</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
@@ -1121,21 +1097,893 @@
         </is>
       </c>
       <c r="J12" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="K12" s="2" t="inlineStr">
+        <is>
+          <t>Fiz uma compra on-line de uma Apostila de Psicologia 2025 e um combo de Aprovação Psico. Já entrei em contato por e-mail, por chat mais não consigo retorno. Já enviei os comprovantes de pagamentos de cada compra, mais não obtenho resposta. Esse material é para concurso, porém a Apostila não abre. Quando clico dá que já foi concluída sem ao menos eu ler. Comprei o material porque preciso, e hoje já entrei e não abre. Gostaria que resolvessem isso. Edna Carvalho</t>
+        </is>
+      </c>
+      <c r="L12" s="2" t="inlineStr">
+        <is>
+          <t>https://www.reclameaqui.com.br/cakto-pay/apostila-de-psicologia-2025-nao-abre-e-cliente-nao-obtem-retorno-sobre-compra-online_30j5btxdpP7LLsjJ/</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>comunidade knights club</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>COMUNIDADE KNIGHTS CLUB</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>angulo</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>Cakto</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>Comunidades / Mentoria de negócios</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>fria</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="H13" s="2" t="inlineStr">
+        <is>
+          <t>R$ 67,99,</t>
+        </is>
+      </c>
+      <c r="I13" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="J13" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="K13" s="2" t="inlineStr">
+        <is>
+          <t>No dia 21/08/2026, realizei a compra da COMUNIDADE KNIGHTS CLUB, no valor de R$ 67,99, através da plataforma de pagamentos Cakto, com pagamento realizado via Pix. Após a compra, descobri que a ferramenta de inteligência artificial adquirida é destinada ao uso em computador. Essa informação não estava suficientemente clara para mim no momento da compra. Como não possuo computador, entrei em contato com o suporte para saber se seria possível utilizar a ferramenta pelo celular e fui informado de qu</t>
+        </is>
+      </c>
+      <c r="L13" s="2" t="inlineStr">
+        <is>
+          <t>https://www.reclameaqui.com.br/cakto-pay/reembolso-de-compra-via-pix-nao-realizado-apos-solicitacao-dentro-do-prazo-legal_w1bmesmQpVhI5h0M/</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>validação cadastral: em análise</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>Validação cadastral: Em análise</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>angulo</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>Cakto</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>Ferramentas de IA / Produtividade</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>fria</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
+          <t>R$ 38,09</t>
+        </is>
+      </c>
+      <c r="I14" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="J14" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="K14" s="2" t="inlineStr">
+        <is>
+          <t>Olá, equipe da Cakto.Estou com um problema sério em relação à validação dos meus documentos na plataforma. Realizei o envio do meu documento digital no dia 18 de agosto, e desde então o status permanece travado como "Validação cadastral: Em análise".Já se passaram semanas e o processo não avança. Por conta dessa demora na análise, não consigo realizar movimentações na minha conta. Atualmente, possuo um saldo de R$ 38,09 categorizado como "Disponível para transferir", mas a opção de "Efetuar Saqu</t>
+        </is>
+      </c>
+      <c r="L14" s="2" t="inlineStr">
+        <is>
+          <t>https://www.reclameaqui.com.br/cakto-pay/demora-na-validacao-de-documentos-impede-movimentacao-e-saque-de-valores-na-plataforma-cakto_AxgK77MKxCN0UISD/</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>continua ativo</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>continua ativo</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>angulo</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>Cakto</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>Infoprodutos - suporte e reembolso</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>fria</t>
+        </is>
+      </c>
+      <c r="G15" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="H15" s="2" t="inlineStr"/>
+      <c r="I15" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="J15" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="K15" s="2" t="inlineStr">
+        <is>
+          <t>O produto continua ativo,sendo que não estou usando o serviço. RA Ads</t>
+        </is>
+      </c>
+      <c r="L15" s="2" t="inlineStr">
+        <is>
+          <t>https://www.reclameaqui.com.br/cakto-pay/cancelamento-de-assinatura-nao-realizado-e-cobranca-indevida-persistente_4mA_vDyxabA5d2h8/</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>manuscrito dos milagres</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>Manuscrito dos Milagres</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>angulo</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>PerfectPay</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>Ferramentas de IA / Produtividade</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>fria</t>
+        </is>
+      </c>
+      <c r="G16" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="H16" s="2" t="inlineStr">
+        <is>
+          <t>R$ 99,00</t>
+        </is>
+      </c>
+      <c r="I16" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="J16" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="K16" s="2" t="inlineStr">
+        <is>
+          <t>Realizei a compra do produto "Manuscrito dos Milagres" no valor de 99 reais através da plataforma de vocês. Trata-se de um [Editado pelo Reclame Aqui] que usa inteligência artificial com a imagem do ator Jonathan Roumie. O conteúdo não foi entregue e não abre. Como estou dentro do prazo legal de 7 dias previsto pelo Artigo 49 do Código de Defesa do Consumidor, exijo o cancelamento imediato e o estorno integral do valor Comprei um produto através da perfectpay Curso(s): Manuscrito dos Milagres Ap</t>
+        </is>
+      </c>
+      <c r="L16" s="2" t="inlineStr">
+        <is>
+          <t>https://www.reclameaqui.com.br/perfectpay/reclamacao-sobre-produto-manuscrito-dos-milagres-nao-entregue-e-solicitacao-de-estorno_YM7HDxei_9htWhyn/</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>youclone no dia 28</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>Youclone no dia 28</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>angulo</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>Cakto</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>Ferramentas de IA / Produtividade</t>
+        </is>
+      </c>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>fria</t>
+        </is>
+      </c>
+      <c r="G17" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="H17" s="2" t="inlineStr">
+        <is>
+          <t>R$ 68,89</t>
+        </is>
+      </c>
+      <c r="I17" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="J17" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="K17" s="2" t="inlineStr">
+        <is>
+          <t>Comprei o produto Youclone no dia 28/08, no pix. Quando fui entrar no curso, não abre a área de membros e não consigo assistir o curso. Na minha área de membros só tem um curso que eu comprei faz tempo. Detalhes do Pedido Pedido: ***** Data: 28/08/2026</t>
+        </is>
+      </c>
+      <c r="L17" s="2" t="inlineStr">
+        <is>
+          <t>https://www.reclameaqui.com.br/cakto-pay/cliente-nao-consegue-acessar-area-de-membros-do-curso-youclone-e-relata-falta-de-suporte_2aC8MLyewmAd3CCU/</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>na ultima quarta feira</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>na ultima quarta feira</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>angulo</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>Cakto</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>Infoprodutos - suporte e reembolso</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
+          <t>fria</t>
+        </is>
+      </c>
+      <c r="G18" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="H18" s="2" t="inlineStr"/>
+      <c r="I18" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="J18" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="K18" s="2" t="inlineStr">
+        <is>
+          <t>Boa noite. Fiz a compra de um produto na ultima quarta feira (26/08/20226) e até essa data eu não recebi o produto. Recebi o e-mail de confirmação do pagamento e um acesso pra fazer o download do material, mas não dá certo. Pra todo lugar que eles me enviam não dá certo. Falo com o pessoal do suporte e eles me deixam sem respostas. Só começam o atendimento. Pedi reembolso, também não dá certo. me mandaram 10 códigos de confirmação e com um segundo diz que expirou. tanto por E-mail quanto por cel</t>
+        </is>
+      </c>
+      <c r="L18" s="2" t="inlineStr">
+        <is>
+          <t>https://www.reclameaqui.com.br/cakto-pay/produto-nao-recebido-e-dificuldade-de-acesso-ao-material-digital-com-falha-no-reembolso-e-suporte-ineficaz_iOzRmbylQ4neQezT/</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>pelo qual paguei n</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>pelo qual paguei n</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>angulo</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>Cakto</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>Ferramentas de IA / Produtividade</t>
+        </is>
+      </c>
+      <c r="F19" s="2" t="inlineStr">
+        <is>
+          <t>fria</t>
+        </is>
+      </c>
+      <c r="G19" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="H19" s="2" t="inlineStr"/>
+      <c r="I19" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="J19" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="K19" s="2" t="inlineStr"/>
+      <c r="L19" s="2" t="inlineStr">
+        <is>
+          <t>https://www.reclameaqui.com.br/cakto-pay/solicitacao-de-reembolso-por-indisponibilidade-do-curso-corselet-classico_kKh1cXRxKbVwJRHp/</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>e conseguiu acess</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>e conseguiu acess</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>angulo</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>Cakto</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>Ferramentas de IA / Produtividade</t>
+        </is>
+      </c>
+      <c r="F20" s="2" t="inlineStr">
+        <is>
+          <t>fria</t>
+        </is>
+      </c>
+      <c r="G20" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="H20" s="2" t="inlineStr">
+        <is>
+          <t>R$ 20,89</t>
+        </is>
+      </c>
+      <c r="I20" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="J20" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="K20" s="2" t="inlineStr"/>
+      <c r="L20" s="2" t="inlineStr">
+        <is>
+          <t>https://www.reclameaqui.com.br/cakto-pay/inconsistencias-na-contabilizacao-de-vendas-e-pagamentos-na-conta-cakto_KtH_3-H9eW4zj_bs/</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>um site hoje e quero solicitar o cancelam</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>um site hoje e quero solicitar o cancelam</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>angulo</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>Cakto</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>Ferramentas de IA / Produtividade</t>
+        </is>
+      </c>
+      <c r="F21" s="2" t="inlineStr">
+        <is>
+          <t>fria</t>
+        </is>
+      </c>
+      <c r="G21" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="H21" s="2" t="inlineStr"/>
+      <c r="I21" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="J21" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="K21" s="2" t="inlineStr"/>
+      <c r="L21" s="2" t="inlineStr">
+        <is>
+          <t>https://www.reclameaqui.com.br/cakto-pay/solicitacao-de-cancelamento-e-estorno-de-3-pedidos-devido-a-arrependimento-e-insatisfacao-com-o-produtosite_KUDEd8s3eGajQ3-L/</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>de seguran</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>de seguran</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>angulo</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>PerfectPay</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>Outros</t>
+        </is>
+      </c>
+      <c r="F22" s="2" t="inlineStr">
+        <is>
+          <t>fria</t>
+        </is>
+      </c>
+      <c r="G22" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="H22" s="2" t="inlineStr"/>
+      <c r="I22" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="J22" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="K22" s="2" t="inlineStr"/>
+      <c r="L22" s="2" t="inlineStr">
+        <is>
+          <t>https://www.reclameaqui.com.br/perfectpay/solicitacao-de-reembolso-de-pedido-com-codigo-de-transacao_poCcMMKbZVAkXZx9/</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>e a plataforma deveria no m</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>e a plataforma deveria no m</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>angulo</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>PerfectPay</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="inlineStr">
+        <is>
+          <t>Ferramentas de IA / Produtividade</t>
+        </is>
+      </c>
+      <c r="F23" s="2" t="inlineStr">
+        <is>
+          <t>fria</t>
+        </is>
+      </c>
+      <c r="G23" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="H23" s="2" t="inlineStr"/>
+      <c r="I23" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="J23" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="K23" s="2" t="inlineStr">
+        <is>
+          <t>Fiz uma compra nessa plataforma e não consigo pedir o reembolso pois a plataforma alega não vender produto. Quero o reembolso pois não gostei do produto e a plataforma deveria no mínimo disponibilizar essa função no site. Segundo a plataforma eu tenho que entrar em contato com o responsável do produto, como irei pedir o reembolso pois o dono do produto não responde. ***** Numero do pedido da minha compra  Reembolso negado por plataforma que alega não vender o produto.</t>
+        </is>
+      </c>
+      <c r="L23" s="2" t="inlineStr">
+        <is>
+          <t>https://www.reclameaqui.com.br/perfectpay/reembolso-negado-por-plataforma-que-alega-nao-vender-o-produto_S-syATG5Z4eLNeZI/</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>stalkeia</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>Stalkeia</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>marca</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>PerfectPay</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t>Espionagem e rastreamento</t>
+        </is>
+      </c>
+      <c r="F24" s="2" t="inlineStr">
+        <is>
+          <t>fria</t>
+        </is>
+      </c>
+      <c r="G24" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="H24" s="2" t="inlineStr">
+        <is>
+          <t>R$ 401,40.</t>
+        </is>
+      </c>
+      <c r="I24" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="J24" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="K24" s="2" t="inlineStr">
+        <is>
+          <t>O produto prometia acesso a contas e mensagens do Instagram, mas na verdade entrega apenas um aplicativo que simula a interface do Instagram e cria conversas artificiais. Ou seja, trata-se de um serviço [Editado pelo Reclame Aqui], que não entrega o que anuncia. Eu testei com dois perfis diferentes e as mensagens são as mesmas, ou seja, [Editado pelo Reclame Aqui] e [Editado pelo Reclame Aqui]. Além disso, após um primeiro pagamento a plataforma vai nos induzindo a efetuar outras compras para co</t>
+        </is>
+      </c>
+      <c r="L24" s="2" t="inlineStr">
+        <is>
+          <t>https://www.reclameaqui.com.br/perfectpay/servico-editado-pelo-reclame-aqui-da-via-perfect-pay-com-promessa-editado-pelo-reclame-aqui_XI7_jZmAIuhQa5In/</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>de postagem autom</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>de postagem autom</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>angulo</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>PerfectPay</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="inlineStr">
+        <is>
+          <t>Espionagem e rastreamento</t>
+        </is>
+      </c>
+      <c r="F25" s="2" t="inlineStr">
+        <is>
+          <t>fria</t>
+        </is>
+      </c>
+      <c r="G25" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="H25" s="2" t="inlineStr"/>
+      <c r="I25" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="J25" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="K25" s="2" t="inlineStr">
+        <is>
+          <t>Comprei um produto ( inteligência artificial com + 10.700 vídeos) com a proposta de postagens automáticas na shopee vídeo, Instagram e tiktok. Porém dentro da plataforma , fui informada que teria que pagar mais um valor para integração com as plataformas, informaram que esse valor é pagamento único, para as plataformas liberarem a integração ( não fica nada com eles). Como meu intuito é as postagens automáticas, comprei. Enviei o comprovante, como solicitado e aguardei o prazo para eles , entrar</t>
+        </is>
+      </c>
+      <c r="L25" s="2" t="inlineStr">
+        <is>
+          <t>https://www.reclameaqui.com.br/perfectpay/reclamacao-sobre-produto-de-postagem-automatica-com-cobrancas-adicionais-sem-retorno-do-suporte-sem-liberacao-do-prometido-e-com-acesso-restrito-ao-conteudoe-falta-de-reembolso_6xa6Ai85fTyG0Yce/</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>uma mentoria no dia 26 onde o reembolso e</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>uma mentoria no dia 26 onde o reembolso e</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>angulo</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>Cakto</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t>Ferramentas de IA / Produtividade</t>
+        </is>
+      </c>
+      <c r="F26" s="2" t="inlineStr">
+        <is>
+          <t>fria</t>
+        </is>
+      </c>
+      <c r="G26" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="H26" s="2" t="inlineStr"/>
+      <c r="I26" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="J26" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="K26" s="2" t="inlineStr">
+        <is>
+          <t>Fiz a compra de uma mentoria no dia 26 onde o reembolso era de responsabilidade do produtor, produtor esse que me ignorou por bastante tempo e disse ter efetuado o reembolso, coisa que eu não sei se aconteceu ou não, por que isso foi antes de ontem e lá na cakto ainda está como "pago" e não algo como "reembolso em andamento" ou coisa assim! Me disseram na última resposta que iam me mandar mensagem no contato cadastrado no reclame aqui, coisa que ainda não fizeram e o prazo pra reembolso é até am</t>
+        </is>
+      </c>
+      <c r="L26" s="2" t="inlineStr">
+        <is>
+          <t>https://www.reclameaqui.com.br/cakto-pay/reclamacao-sobre-reembolso-de-mentoria-nao-processado-e-falta-de-suporte_nV8WPHM4qJbjnUSu/</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>adquirido teria condi</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>adquirido teria condi</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>angulo</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t>Cakto</t>
+        </is>
+      </c>
+      <c r="E27" s="2" t="inlineStr">
+        <is>
+          <t>Ferramentas de IA / Produtividade</t>
+        </is>
+      </c>
+      <c r="F27" s="2" t="inlineStr">
+        <is>
+          <t>fria</t>
+        </is>
+      </c>
+      <c r="G27" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="H27" s="2" t="inlineStr"/>
+      <c r="I27" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="J27" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="K27" s="2" t="inlineStr">
+        <is>
+          <t>Venho solicitar a contestação de uma compra realizada referente à contratação de uma estrutura montada para geração de retorno financeiro. A contratação foi realizada acreditando que o serviço/produto adquirido teria condições de funcionar conforme apresentado pelos responsáveis pela estrutura. O problema é que, após a contratação e a montagem das estruturas, o resultado esperado não aconteceu. Além do valor já pago pela aquisição do produto/estrutura, posteriormente fui informado de que seria n</t>
+        </is>
+      </c>
+      <c r="L27" s="2" t="inlineStr">
+        <is>
+          <t>https://www.reclameaqui.com.br/cakto-pay/contestacao-de-compra-de-estrutura-para-geracao-de-retorno-financeiro-nao-concretizado-e-falta-de-informacao-sobre-investimentos-adicionais_CUW1-e-tTFELAg9M/</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>dois cursos de idiomas</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>dois cursos de idiomas</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>angulo</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t>Cakto</t>
+        </is>
+      </c>
+      <c r="E28" s="2" t="inlineStr">
+        <is>
+          <t>Ferramentas de IA / Produtividade</t>
+        </is>
+      </c>
+      <c r="F28" s="2" t="inlineStr">
+        <is>
+          <t>fria</t>
+        </is>
+      </c>
+      <c r="G28" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="H28" s="2" t="inlineStr"/>
+      <c r="I28" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="J28" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="K12" s="2" t="inlineStr">
-        <is>
-          <t>Veja também todas as reclamações não respondidas respondidas finalizadas Apostila de Psicologia 2025 não abre e cliente não obtém retorno sobre compra online.  Respondida  CAKTO PAY  Sorocaba - SP  01/09/2026 às 10:19  ID: 257909223  Fiz uma compra on-line de uma Apostila de Psicologia 2025 e um com</t>
-        </is>
-      </c>
-      <c r="L12" s="2" t="inlineStr">
-        <is>
-          <t>https://www.reclameaqui.com.br/cakto-pay/apostila-de-psicologia-2025-nao-abre-e-cliente-nao-obtem-retorno-sobre-compra-online_30j5btxdpP7LLsjJ/</t>
+      <c r="K28" s="2" t="inlineStr">
+        <is>
+          <t>Fiz uma compra de dois cursos de idiomas, no caso Espanhol. Paguei pelos dois cursos via pi, porém só tive acesso a um curso, o outro aparece como acesso negado e não consigo acessar. Já entrei em contato com o suporte, porém o email retorna como email inválido. Entro em contato com o suporte para solicitar reembolso e ninguém me dá um retorno. Solicito devolução do valor, porém não tenho contato com ninguém da empresa. Acesso negado a curso de espanhol pago e dificuldade de contato com o suport</t>
+        </is>
+      </c>
+      <c r="L28" s="2" t="inlineStr">
+        <is>
+          <t>https://www.reclameaqui.com.br/cakto-pay/acesso-negado-a-curso-de-espanhol-pago-e-dificuldade-de-contato-com-o-suporte-para-reembolso_9d9eJH4OMC_ApZLR/</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L12"/>
+  <autoFilter ref="A1:L28"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1146,7 +1994,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G5"/>
+  <dimension ref="A1:G13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -1202,13 +2050,13 @@
         </is>
       </c>
       <c r="B2" s="4" t="n">
-        <v>4</v>
+        <v>12</v>
       </c>
       <c r="C2" s="4" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D2" s="4" t="n">
-        <v>2</v>
+        <v>12</v>
       </c>
       <c r="E2" s="4" t="n">
         <v>0</v>
@@ -1217,7 +2065,7 @@
         <v>0</v>
       </c>
       <c r="G2" s="4" t="n">
-        <v>4</v>
+        <v>12</v>
       </c>
     </row>
     <row r="3">
@@ -1227,14 +2075,14 @@
         </is>
       </c>
       <c r="B3" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="C3" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="D3" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="C3" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="D3" s="4" t="n">
-        <v>0</v>
-      </c>
       <c r="E3" s="4" t="n">
         <v>0</v>
       </c>
@@ -1242,24 +2090,24 @@
         <v>0</v>
       </c>
       <c r="G3" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
         <is>
-          <t>Educação e consultoria</t>
+          <t>Infoprodutos - suporte e reembolso</t>
         </is>
       </c>
       <c r="B4" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C4" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D4" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="D4" s="4" t="n">
-        <v>1</v>
-      </c>
       <c r="E4" s="4" t="n">
         <v>0</v>
       </c>
@@ -1267,23 +2115,23 @@
         <v>0</v>
       </c>
       <c r="G4" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>Ganhar dinheiro online / trabalho remoto</t>
+          <t>Educação / Marketing digital e low ticket</t>
         </is>
       </c>
       <c r="B5" s="4" t="n">
         <v>1</v>
       </c>
       <c r="C5" s="4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D5" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E5" s="4" t="n">
         <v>0</v>
@@ -1292,6 +2140,206 @@
         <v>0</v>
       </c>
       <c r="G5" s="4" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>Educação e consultoria</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="C6" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="D6" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E6" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F6" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G6" s="4" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>Ferramentas de IA / Cloaking</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="C7" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D7" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="E7" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F7" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G7" s="4" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>Ganhar dinheiro online / Ferramentas de afiliado</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="C8" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D8" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="E8" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F8" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G8" s="4" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>Produtos digitais variados / Assinatura vitalícia</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="C9" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D9" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="E9" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F9" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G9" s="4" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>Ferramentas de espionagem / WhatsApp</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="C10" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D10" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="E10" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F10" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G10" s="4" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>Educação / Concursos e certificações</t>
+        </is>
+      </c>
+      <c r="B11" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="C11" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D11" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="E11" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F11" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G11" s="4" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>Comunidades / Mentoria de negócios</t>
+        </is>
+      </c>
+      <c r="B12" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="C12" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D12" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="E12" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F12" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G12" s="4" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>Outros</t>
+        </is>
+      </c>
+      <c r="B13" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="C13" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D13" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="E13" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F13" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G13" s="4" t="n">
         <v>1</v>
       </c>
     </row>
@@ -1373,7 +2421,7 @@
         </is>
       </c>
       <c r="C4" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="5">
@@ -1433,7 +2481,7 @@
         </is>
       </c>
       <c r="C8" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="9">
@@ -1463,7 +2511,7 @@
         </is>
       </c>
       <c r="C10" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="11">
@@ -1568,7 +2616,7 @@
         </is>
       </c>
       <c r="C17" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="18">
@@ -1598,7 +2646,7 @@
         </is>
       </c>
       <c r="C19" s="4" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="20">
@@ -1718,7 +2766,7 @@
         </is>
       </c>
       <c r="C27" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="28">
@@ -1748,7 +2796,7 @@
         </is>
       </c>
       <c r="C29" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="30">
@@ -1763,7 +2811,7 @@
         </is>
       </c>
       <c r="C30" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="31">
@@ -1778,7 +2826,7 @@
         </is>
       </c>
       <c r="C31" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="32">
@@ -1793,7 +2841,7 @@
         </is>
       </c>
       <c r="C32" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="33">
@@ -1868,7 +2916,7 @@
         </is>
       </c>
       <c r="C37" s="4" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
radar 2026-09-03: +0 novas, 0 atualizadas, 0 snapshots
</commit_message>
<xml_diff>
--- a/Radar/radar-low-ticket.xlsx
+++ b/Radar/radar-low-ticket.xlsx
@@ -565,7 +565,7 @@
         </is>
       </c>
       <c r="J2" s="2" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="K2" s="2" t="inlineStr">
         <is>
@@ -619,7 +619,7 @@
         </is>
       </c>
       <c r="J3" s="2" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
@@ -673,7 +673,7 @@
         </is>
       </c>
       <c r="J4" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K4" s="2" t="inlineStr">
         <is>
@@ -731,7 +731,7 @@
         </is>
       </c>
       <c r="J5" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K5" s="2" t="inlineStr">
         <is>
@@ -785,7 +785,7 @@
         </is>
       </c>
       <c r="J6" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K6" s="2" t="inlineStr"/>
       <c r="L6" s="2" t="inlineStr">
@@ -839,7 +839,7 @@
         </is>
       </c>
       <c r="J7" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K7" s="2" t="inlineStr">
         <is>
@@ -893,7 +893,7 @@
         </is>
       </c>
       <c r="J8" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K8" s="2" t="inlineStr"/>
       <c r="L8" s="2" t="inlineStr">
@@ -943,7 +943,7 @@
         </is>
       </c>
       <c r="J9" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K9" s="2" t="inlineStr">
         <is>
@@ -1001,7 +1001,7 @@
         </is>
       </c>
       <c r="J10" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K10" s="2" t="inlineStr">
         <is>
@@ -1055,7 +1055,7 @@
         </is>
       </c>
       <c r="J11" s="2" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="K11" s="2" t="inlineStr">
         <is>
@@ -1113,7 +1113,7 @@
         </is>
       </c>
       <c r="J12" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K12" s="2" t="inlineStr">
         <is>
@@ -1167,7 +1167,7 @@
         </is>
       </c>
       <c r="J13" s="2" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="K13" s="2" t="inlineStr">
         <is>
@@ -1221,7 +1221,7 @@
         </is>
       </c>
       <c r="J14" s="2" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="K14" s="2" t="inlineStr">
         <is>
@@ -1275,7 +1275,7 @@
         </is>
       </c>
       <c r="J15" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K15" s="2" t="inlineStr">
         <is>
@@ -1333,7 +1333,7 @@
         </is>
       </c>
       <c r="J16" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K16" s="2" t="inlineStr"/>
       <c r="L16" s="2" t="inlineStr">
@@ -1383,7 +1383,7 @@
         </is>
       </c>
       <c r="J17" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K17" s="2" t="inlineStr">
         <is>
@@ -1437,7 +1437,7 @@
         </is>
       </c>
       <c r="J18" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K18" s="2" t="inlineStr">
         <is>
@@ -1491,7 +1491,7 @@
         </is>
       </c>
       <c r="J19" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K19" s="2" t="inlineStr">
         <is>
@@ -1545,7 +1545,7 @@
         </is>
       </c>
       <c r="J20" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K20" s="2" t="inlineStr">
         <is>
@@ -1599,7 +1599,7 @@
         </is>
       </c>
       <c r="J21" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K21" s="2" t="inlineStr"/>
       <c r="L21" s="2" t="inlineStr">
@@ -1649,7 +1649,7 @@
         </is>
       </c>
       <c r="J22" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K22" s="2" t="inlineStr">
         <is>
@@ -1703,7 +1703,7 @@
         </is>
       </c>
       <c r="J23" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K23" s="2" t="inlineStr">
         <is>
@@ -1757,7 +1757,7 @@
         </is>
       </c>
       <c r="J24" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K24" s="2" t="inlineStr"/>
       <c r="L24" s="2" t="inlineStr">
@@ -1807,7 +1807,7 @@
         </is>
       </c>
       <c r="J25" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K25" s="2" t="inlineStr">
         <is>
@@ -1861,7 +1861,7 @@
         </is>
       </c>
       <c r="J26" s="2" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="K26" s="2" t="inlineStr">
         <is>
@@ -1915,7 +1915,7 @@
         </is>
       </c>
       <c r="J27" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K27" s="2" t="inlineStr"/>
       <c r="L27" s="2" t="inlineStr">
@@ -1965,7 +1965,7 @@
         </is>
       </c>
       <c r="J28" s="2" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="K28" s="2" t="inlineStr"/>
       <c r="L28" s="2" t="inlineStr">
@@ -2015,7 +2015,7 @@
         </is>
       </c>
       <c r="J29" s="2" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="K29" s="2" t="inlineStr">
         <is>
@@ -2069,7 +2069,7 @@
         </is>
       </c>
       <c r="J30" s="2" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="K30" s="2" t="inlineStr"/>
       <c r="L30" s="2" t="inlineStr">
@@ -2119,7 +2119,7 @@
         </is>
       </c>
       <c r="J31" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K31" s="2" t="inlineStr"/>
       <c r="L31" s="2" t="inlineStr">
@@ -2169,7 +2169,7 @@
         </is>
       </c>
       <c r="J32" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K32" s="2" t="inlineStr">
         <is>
@@ -2223,7 +2223,7 @@
         </is>
       </c>
       <c r="J33" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K33" s="2" t="inlineStr">
         <is>
@@ -2277,7 +2277,7 @@
         </is>
       </c>
       <c r="J34" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K34" s="2" t="inlineStr">
         <is>
@@ -2331,7 +2331,7 @@
         </is>
       </c>
       <c r="J35" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K35" s="2" t="inlineStr"/>
       <c r="L35" s="2" t="inlineStr">
@@ -2381,7 +2381,7 @@
         </is>
       </c>
       <c r="J36" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K36" s="2" t="inlineStr"/>
       <c r="L36" s="2" t="inlineStr">
@@ -2431,7 +2431,7 @@
         </is>
       </c>
       <c r="J37" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K37" s="2" t="inlineStr">
         <is>
@@ -2485,7 +2485,7 @@
         </is>
       </c>
       <c r="J38" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K38" s="2" t="inlineStr">
         <is>
@@ -2539,7 +2539,7 @@
         </is>
       </c>
       <c r="J39" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K39" s="2" t="inlineStr">
         <is>
@@ -2593,7 +2593,7 @@
         </is>
       </c>
       <c r="J40" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K40" s="2" t="inlineStr"/>
       <c r="L40" s="2" t="inlineStr">
@@ -2643,7 +2643,7 @@
         </is>
       </c>
       <c r="J41" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K41" s="2" t="inlineStr">
         <is>
@@ -2697,7 +2697,7 @@
         </is>
       </c>
       <c r="J42" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K42" s="2" t="inlineStr"/>
       <c r="L42" s="2" t="inlineStr">
@@ -2751,7 +2751,7 @@
         </is>
       </c>
       <c r="J43" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K43" s="2" t="inlineStr">
         <is>
@@ -2805,7 +2805,7 @@
         </is>
       </c>
       <c r="J44" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K44" s="2" t="inlineStr">
         <is>
@@ -2859,7 +2859,7 @@
         </is>
       </c>
       <c r="J45" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K45" s="2" t="inlineStr">
         <is>
@@ -2913,7 +2913,7 @@
         </is>
       </c>
       <c r="J46" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K46" s="2" t="inlineStr">
         <is>
@@ -2967,7 +2967,7 @@
         </is>
       </c>
       <c r="J47" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K47" s="2" t="inlineStr">
         <is>
@@ -3021,7 +3021,7 @@
         </is>
       </c>
       <c r="J48" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K48" s="2" t="inlineStr">
         <is>
@@ -3075,7 +3075,7 @@
         </is>
       </c>
       <c r="J49" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K49" s="2" t="inlineStr">
         <is>
@@ -3129,7 +3129,7 @@
         </is>
       </c>
       <c r="J50" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K50" s="2" t="inlineStr">
         <is>
@@ -3183,7 +3183,7 @@
         </is>
       </c>
       <c r="J51" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K51" s="2" t="inlineStr">
         <is>
@@ -3237,7 +3237,7 @@
         </is>
       </c>
       <c r="J52" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K52" s="2" t="inlineStr">
         <is>
@@ -3291,7 +3291,7 @@
         </is>
       </c>
       <c r="J53" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K53" s="2" t="inlineStr">
         <is>
@@ -3345,7 +3345,7 @@
         </is>
       </c>
       <c r="J54" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K54" s="2" t="inlineStr">
         <is>
@@ -3399,7 +3399,7 @@
         </is>
       </c>
       <c r="J55" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K55" s="2" t="inlineStr">
         <is>
@@ -3453,7 +3453,7 @@
         </is>
       </c>
       <c r="J56" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K56" s="2" t="inlineStr">
         <is>
@@ -3507,7 +3507,7 @@
         </is>
       </c>
       <c r="J57" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K57" s="2" t="inlineStr">
         <is>
@@ -3561,7 +3561,7 @@
         </is>
       </c>
       <c r="J58" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K58" s="2" t="inlineStr"/>
       <c r="L58" s="2" t="inlineStr">
@@ -3611,7 +3611,7 @@
         </is>
       </c>
       <c r="J59" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K59" s="2" t="inlineStr">
         <is>
@@ -3665,7 +3665,7 @@
         </is>
       </c>
       <c r="J60" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K60" s="2" t="inlineStr">
         <is>
@@ -3719,7 +3719,7 @@
         </is>
       </c>
       <c r="J61" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K61" s="2" t="inlineStr">
         <is>
@@ -3773,7 +3773,7 @@
         </is>
       </c>
       <c r="J62" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K62" s="2" t="inlineStr"/>
       <c r="L62" s="2" t="inlineStr">
@@ -3823,7 +3823,7 @@
         </is>
       </c>
       <c r="J63" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K63" s="2" t="inlineStr"/>
       <c r="L63" s="2" t="inlineStr">
@@ -3873,7 +3873,7 @@
         </is>
       </c>
       <c r="J64" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K64" s="2" t="inlineStr">
         <is>
@@ -3927,7 +3927,7 @@
         </is>
       </c>
       <c r="J65" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K65" s="2" t="inlineStr">
         <is>
@@ -3981,7 +3981,7 @@
         </is>
       </c>
       <c r="J66" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K66" s="2" t="inlineStr">
         <is>
@@ -4035,7 +4035,7 @@
         </is>
       </c>
       <c r="J67" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K67" s="2" t="inlineStr"/>
       <c r="L67" s="2" t="inlineStr">
@@ -4085,7 +4085,7 @@
         </is>
       </c>
       <c r="J68" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K68" s="2" t="inlineStr"/>
       <c r="L68" s="2" t="inlineStr">
@@ -4135,7 +4135,7 @@
         </is>
       </c>
       <c r="J69" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K69" s="2" t="inlineStr"/>
       <c r="L69" s="2" t="inlineStr">
@@ -4185,7 +4185,7 @@
         </is>
       </c>
       <c r="J70" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K70" s="2" t="inlineStr">
         <is>
@@ -4239,7 +4239,7 @@
         </is>
       </c>
       <c r="J71" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K71" s="2" t="inlineStr"/>
       <c r="L71" s="2" t="inlineStr">
@@ -4289,7 +4289,7 @@
         </is>
       </c>
       <c r="J72" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K72" s="2" t="inlineStr">
         <is>
@@ -4347,7 +4347,7 @@
         </is>
       </c>
       <c r="J73" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K73" s="2" t="inlineStr">
         <is>
@@ -4405,7 +4405,7 @@
         </is>
       </c>
       <c r="J74" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K74" s="2" t="inlineStr">
         <is>
@@ -4459,7 +4459,7 @@
         </is>
       </c>
       <c r="J75" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K75" s="2" t="inlineStr">
         <is>
@@ -4513,7 +4513,7 @@
         </is>
       </c>
       <c r="J76" s="2" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="K76" s="2" t="inlineStr">
         <is>
@@ -4567,7 +4567,7 @@
         </is>
       </c>
       <c r="J77" s="2" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="K77" s="2" t="inlineStr">
         <is>
@@ -4621,7 +4621,7 @@
         </is>
       </c>
       <c r="J78" s="2" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="K78" s="2" t="inlineStr">
         <is>
@@ -4675,7 +4675,7 @@
         </is>
       </c>
       <c r="J79" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K79" s="2" t="inlineStr"/>
       <c r="L79" s="2" t="inlineStr">
@@ -4725,7 +4725,7 @@
         </is>
       </c>
       <c r="J80" s="2" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="K80" s="2" t="inlineStr">
         <is>
@@ -4779,7 +4779,7 @@
         </is>
       </c>
       <c r="J81" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K81" s="2" t="inlineStr">
         <is>
@@ -4833,7 +4833,7 @@
         </is>
       </c>
       <c r="J82" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K82" s="2" t="inlineStr">
         <is>
@@ -4887,7 +4887,7 @@
         </is>
       </c>
       <c r="J83" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K83" s="2" t="inlineStr"/>
       <c r="L83" s="2" t="inlineStr">
@@ -4937,7 +4937,7 @@
         </is>
       </c>
       <c r="J84" s="2" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="K84" s="2" t="inlineStr">
         <is>
@@ -4991,7 +4991,7 @@
         </is>
       </c>
       <c r="J85" s="2" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="K85" s="2" t="inlineStr">
         <is>
@@ -5045,7 +5045,7 @@
         </is>
       </c>
       <c r="J86" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K86" s="2" t="inlineStr">
         <is>
@@ -5099,7 +5099,7 @@
         </is>
       </c>
       <c r="J87" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K87" s="2" t="inlineStr"/>
       <c r="L87" s="2" t="inlineStr">
@@ -5149,7 +5149,7 @@
         </is>
       </c>
       <c r="J88" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K88" s="2" t="inlineStr"/>
       <c r="L88" s="2" t="inlineStr">
@@ -5199,7 +5199,7 @@
         </is>
       </c>
       <c r="J89" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K89" s="2" t="inlineStr">
         <is>
@@ -5253,7 +5253,7 @@
         </is>
       </c>
       <c r="J90" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K90" s="2" t="inlineStr">
         <is>
@@ -5307,7 +5307,7 @@
         </is>
       </c>
       <c r="J91" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K91" s="2" t="inlineStr"/>
       <c r="L91" s="2" t="inlineStr">
@@ -5357,7 +5357,7 @@
         </is>
       </c>
       <c r="J92" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K92" s="2" t="inlineStr">
         <is>
@@ -5411,7 +5411,7 @@
         </is>
       </c>
       <c r="J93" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K93" s="2" t="inlineStr">
         <is>
@@ -5465,7 +5465,7 @@
         </is>
       </c>
       <c r="J94" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K94" s="2" t="inlineStr">
         <is>
@@ -5519,7 +5519,7 @@
         </is>
       </c>
       <c r="J95" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K95" s="2" t="inlineStr">
         <is>
@@ -5573,7 +5573,7 @@
         </is>
       </c>
       <c r="J96" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K96" s="2" t="inlineStr"/>
       <c r="L96" s="2" t="inlineStr">
@@ -5623,7 +5623,7 @@
         </is>
       </c>
       <c r="J97" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K97" s="2" t="inlineStr">
         <is>
@@ -5677,7 +5677,7 @@
         </is>
       </c>
       <c r="J98" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K98" s="2" t="inlineStr">
         <is>
@@ -5731,7 +5731,7 @@
         </is>
       </c>
       <c r="J99" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K99" s="2" t="inlineStr">
         <is>
@@ -5785,7 +5785,7 @@
         </is>
       </c>
       <c r="J100" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K100" s="2" t="inlineStr"/>
       <c r="L100" s="2" t="inlineStr">
@@ -5835,7 +5835,7 @@
         </is>
       </c>
       <c r="J101" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K101" s="2" t="inlineStr"/>
       <c r="L101" s="2" t="inlineStr">
@@ -5885,7 +5885,7 @@
         </is>
       </c>
       <c r="J102" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K102" s="2" t="inlineStr">
         <is>
@@ -5939,7 +5939,7 @@
         </is>
       </c>
       <c r="J103" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K103" s="2" t="inlineStr">
         <is>
@@ -5993,7 +5993,7 @@
         </is>
       </c>
       <c r="J104" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K104" s="2" t="inlineStr">
         <is>
@@ -6690,7 +6690,7 @@
         </is>
       </c>
       <c r="C2" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="3">
@@ -6720,7 +6720,7 @@
         </is>
       </c>
       <c r="C4" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="5">
@@ -6735,7 +6735,7 @@
         </is>
       </c>
       <c r="C5" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="6">
@@ -6765,7 +6765,7 @@
         </is>
       </c>
       <c r="C7" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="8">
@@ -6780,7 +6780,7 @@
         </is>
       </c>
       <c r="C8" s="4" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="9">
@@ -6825,7 +6825,7 @@
         </is>
       </c>
       <c r="C11" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="12">
@@ -6840,7 +6840,7 @@
         </is>
       </c>
       <c r="C12" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="13">
@@ -6855,7 +6855,7 @@
         </is>
       </c>
       <c r="C13" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="14">
@@ -6870,7 +6870,7 @@
         </is>
       </c>
       <c r="C14" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="15">
@@ -6885,7 +6885,7 @@
         </is>
       </c>
       <c r="C15" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="16">
@@ -6915,7 +6915,7 @@
         </is>
       </c>
       <c r="C17" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="18">
@@ -6930,7 +6930,7 @@
         </is>
       </c>
       <c r="C18" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="19">
@@ -6945,7 +6945,7 @@
         </is>
       </c>
       <c r="C19" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="20">
@@ -6960,7 +6960,7 @@
         </is>
       </c>
       <c r="C20" s="4" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="21">
@@ -6975,7 +6975,7 @@
         </is>
       </c>
       <c r="C21" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="22">
@@ -6990,7 +6990,7 @@
         </is>
       </c>
       <c r="C22" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="23">
@@ -7020,7 +7020,7 @@
         </is>
       </c>
       <c r="C24" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="25">
@@ -7035,7 +7035,7 @@
         </is>
       </c>
       <c r="C25" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="26">
@@ -7050,7 +7050,7 @@
         </is>
       </c>
       <c r="C26" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="27">
@@ -7065,7 +7065,7 @@
         </is>
       </c>
       <c r="C27" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="28">
@@ -7080,7 +7080,7 @@
         </is>
       </c>
       <c r="C28" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="29">
@@ -7095,7 +7095,7 @@
         </is>
       </c>
       <c r="C29" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="30">
@@ -7110,7 +7110,7 @@
         </is>
       </c>
       <c r="C30" s="4" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="31">
@@ -7125,7 +7125,7 @@
         </is>
       </c>
       <c r="C31" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="32">
@@ -7140,7 +7140,7 @@
         </is>
       </c>
       <c r="C32" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="33">
@@ -7155,7 +7155,7 @@
         </is>
       </c>
       <c r="C33" s="4" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="34">
@@ -7185,7 +7185,7 @@
         </is>
       </c>
       <c r="C35" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="36">
@@ -7200,7 +7200,7 @@
         </is>
       </c>
       <c r="C36" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="37">
@@ -7215,7 +7215,7 @@
         </is>
       </c>
       <c r="C37" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="38">
@@ -7230,7 +7230,7 @@
         </is>
       </c>
       <c r="C38" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="39">
@@ -7245,7 +7245,7 @@
         </is>
       </c>
       <c r="C39" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="40">
@@ -7260,7 +7260,7 @@
         </is>
       </c>
       <c r="C40" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="41">
@@ -7275,7 +7275,7 @@
         </is>
       </c>
       <c r="C41" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="42">
@@ -7335,7 +7335,7 @@
         </is>
       </c>
       <c r="C45" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="46">
@@ -7350,7 +7350,7 @@
         </is>
       </c>
       <c r="C46" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="47">
@@ -7365,7 +7365,7 @@
         </is>
       </c>
       <c r="C47" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="48">
@@ -7380,7 +7380,7 @@
         </is>
       </c>
       <c r="C48" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="49">
@@ -7395,7 +7395,7 @@
         </is>
       </c>
       <c r="C49" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="50">
@@ -7410,7 +7410,7 @@
         </is>
       </c>
       <c r="C50" s="4" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="51">
@@ -7425,7 +7425,7 @@
         </is>
       </c>
       <c r="C51" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="52">
@@ -7440,7 +7440,7 @@
         </is>
       </c>
       <c r="C52" s="4" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="53">
@@ -7455,7 +7455,7 @@
         </is>
       </c>
       <c r="C53" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="54">
@@ -7470,7 +7470,7 @@
         </is>
       </c>
       <c r="C54" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="55">
@@ -7485,7 +7485,7 @@
         </is>
       </c>
       <c r="C55" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="56">
@@ -7500,7 +7500,7 @@
         </is>
       </c>
       <c r="C56" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="57">
@@ -7545,7 +7545,7 @@
         </is>
       </c>
       <c r="C59" s="4" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="60">
@@ -7575,7 +7575,7 @@
         </is>
       </c>
       <c r="C61" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="62">
@@ -7590,7 +7590,7 @@
         </is>
       </c>
       <c r="C62" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="63">
@@ -7605,7 +7605,7 @@
         </is>
       </c>
       <c r="C63" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="64">
@@ -7620,7 +7620,7 @@
         </is>
       </c>
       <c r="C64" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="65">
@@ -7635,7 +7635,7 @@
         </is>
       </c>
       <c r="C65" s="4" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="66">
@@ -7650,7 +7650,7 @@
         </is>
       </c>
       <c r="C66" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="67">
@@ -7665,7 +7665,7 @@
         </is>
       </c>
       <c r="C67" s="4" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="68">
@@ -7680,7 +7680,7 @@
         </is>
       </c>
       <c r="C68" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="69">
@@ -7695,7 +7695,7 @@
         </is>
       </c>
       <c r="C69" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="70">
@@ -7710,7 +7710,7 @@
         </is>
       </c>
       <c r="C70" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="71">
@@ -7725,7 +7725,7 @@
         </is>
       </c>
       <c r="C71" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="72">
@@ -7755,7 +7755,7 @@
         </is>
       </c>
       <c r="C73" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="74">
@@ -7785,7 +7785,7 @@
         </is>
       </c>
       <c r="C75" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="76">
@@ -7800,7 +7800,7 @@
         </is>
       </c>
       <c r="C76" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="77">
@@ -7830,7 +7830,7 @@
         </is>
       </c>
       <c r="C78" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="79">
@@ -7845,7 +7845,7 @@
         </is>
       </c>
       <c r="C79" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="80">
@@ -7875,7 +7875,7 @@
         </is>
       </c>
       <c r="C81" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="82">
@@ -7890,7 +7890,7 @@
         </is>
       </c>
       <c r="C82" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="83">
@@ -7905,7 +7905,7 @@
         </is>
       </c>
       <c r="C83" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="84">
@@ -7920,7 +7920,7 @@
         </is>
       </c>
       <c r="C84" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="85">
@@ -7935,7 +7935,7 @@
         </is>
       </c>
       <c r="C85" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="86">
@@ -7950,7 +7950,7 @@
         </is>
       </c>
       <c r="C86" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="87">
@@ -7965,7 +7965,7 @@
         </is>
       </c>
       <c r="C87" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="88">
@@ -7980,7 +7980,7 @@
         </is>
       </c>
       <c r="C88" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="89">
@@ -8010,7 +8010,7 @@
         </is>
       </c>
       <c r="C90" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="91">
@@ -8025,7 +8025,7 @@
         </is>
       </c>
       <c r="C91" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="92">
@@ -8040,7 +8040,7 @@
         </is>
       </c>
       <c r="C92" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="93">
@@ -8055,7 +8055,7 @@
         </is>
       </c>
       <c r="C93" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="94">
@@ -8070,7 +8070,7 @@
         </is>
       </c>
       <c r="C94" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="95">
@@ -8085,7 +8085,7 @@
         </is>
       </c>
       <c r="C95" s="4" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="96">
@@ -8100,7 +8100,7 @@
         </is>
       </c>
       <c r="C96" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="97">
@@ -8115,7 +8115,7 @@
         </is>
       </c>
       <c r="C97" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="98">
@@ -8130,7 +8130,7 @@
         </is>
       </c>
       <c r="C98" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="99">
@@ -8145,7 +8145,7 @@
         </is>
       </c>
       <c r="C99" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="100">
@@ -8160,7 +8160,7 @@
         </is>
       </c>
       <c r="C100" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="101">
@@ -8175,7 +8175,7 @@
         </is>
       </c>
       <c r="C101" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="102">
@@ -8190,7 +8190,7 @@
         </is>
       </c>
       <c r="C102" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="103">
@@ -8205,7 +8205,7 @@
         </is>
       </c>
       <c r="C103" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="104">
@@ -8220,7 +8220,7 @@
         </is>
       </c>
       <c r="C104" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="105">
@@ -8235,7 +8235,7 @@
         </is>
       </c>
       <c r="C105" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="106">
@@ -8265,7 +8265,7 @@
         </is>
       </c>
       <c r="C107" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="108">
@@ -8280,7 +8280,7 @@
         </is>
       </c>
       <c r="C108" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="109">
@@ -8295,7 +8295,7 @@
         </is>
       </c>
       <c r="C109" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="110">
@@ -8310,7 +8310,7 @@
         </is>
       </c>
       <c r="C110" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="111">
@@ -8325,7 +8325,7 @@
         </is>
       </c>
       <c r="C111" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="112">
@@ -8340,7 +8340,7 @@
         </is>
       </c>
       <c r="C112" s="4" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="113">
@@ -8355,7 +8355,7 @@
         </is>
       </c>
       <c r="C113" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="114">
@@ -8370,7 +8370,7 @@
         </is>
       </c>
       <c r="C114" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="115">
@@ -8385,7 +8385,7 @@
         </is>
       </c>
       <c r="C115" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="116">
@@ -8400,7 +8400,7 @@
         </is>
       </c>
       <c r="C116" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="117">
@@ -8415,7 +8415,7 @@
         </is>
       </c>
       <c r="C117" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="118">
@@ -8430,7 +8430,7 @@
         </is>
       </c>
       <c r="C118" s="4" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="119">
@@ -8445,7 +8445,7 @@
         </is>
       </c>
       <c r="C119" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="120">
@@ -8460,7 +8460,7 @@
         </is>
       </c>
       <c r="C120" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="121">
@@ -8490,7 +8490,7 @@
         </is>
       </c>
       <c r="C122" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="123">
@@ -8505,7 +8505,7 @@
         </is>
       </c>
       <c r="C123" s="4" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="124">
@@ -8520,7 +8520,7 @@
         </is>
       </c>
       <c r="C124" s="4" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
radar 2026-09-04: +0 novas, 0 atualizadas, 0 snapshots
</commit_message>
<xml_diff>
--- a/Radar/radar-low-ticket.xlsx
+++ b/Radar/radar-low-ticket.xlsx
@@ -565,7 +565,7 @@
         </is>
       </c>
       <c r="J2" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K2" s="2" t="inlineStr">
         <is>
@@ -619,7 +619,7 @@
         </is>
       </c>
       <c r="J3" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
@@ -673,7 +673,7 @@
         </is>
       </c>
       <c r="J4" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K4" s="2" t="inlineStr">
         <is>
@@ -727,7 +727,7 @@
         </is>
       </c>
       <c r="J5" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K5" s="2" t="inlineStr">
         <is>
@@ -785,7 +785,7 @@
         </is>
       </c>
       <c r="J6" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K6" s="2" t="inlineStr">
         <is>
@@ -839,7 +839,7 @@
         </is>
       </c>
       <c r="J7" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K7" s="2" t="inlineStr"/>
       <c r="L7" s="2" t="inlineStr">
@@ -893,7 +893,7 @@
         </is>
       </c>
       <c r="J8" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K8" s="2" t="inlineStr">
         <is>
@@ -947,7 +947,7 @@
         </is>
       </c>
       <c r="J9" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K9" s="2" t="inlineStr"/>
       <c r="L9" s="2" t="inlineStr">
@@ -997,7 +997,7 @@
         </is>
       </c>
       <c r="J10" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K10" s="2" t="inlineStr">
         <is>
@@ -1055,7 +1055,7 @@
         </is>
       </c>
       <c r="J11" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K11" s="2" t="inlineStr">
         <is>
@@ -1109,7 +1109,7 @@
         </is>
       </c>
       <c r="J12" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K12" s="2" t="inlineStr">
         <is>
@@ -1167,7 +1167,7 @@
         </is>
       </c>
       <c r="J13" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K13" s="2" t="inlineStr">
         <is>
@@ -1221,7 +1221,7 @@
         </is>
       </c>
       <c r="J14" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K14" s="2" t="inlineStr">
         <is>
@@ -1275,7 +1275,7 @@
         </is>
       </c>
       <c r="J15" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K15" s="2" t="inlineStr">
         <is>
@@ -1329,7 +1329,7 @@
         </is>
       </c>
       <c r="J16" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K16" s="2" t="inlineStr">
         <is>
@@ -1387,7 +1387,7 @@
         </is>
       </c>
       <c r="J17" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K17" s="2" t="inlineStr"/>
       <c r="L17" s="2" t="inlineStr">
@@ -1437,7 +1437,7 @@
         </is>
       </c>
       <c r="J18" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K18" s="2" t="inlineStr">
         <is>
@@ -1491,7 +1491,7 @@
         </is>
       </c>
       <c r="J19" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K19" s="2" t="inlineStr">
         <is>
@@ -1545,7 +1545,7 @@
         </is>
       </c>
       <c r="J20" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K20" s="2" t="inlineStr">
         <is>
@@ -1599,7 +1599,7 @@
         </is>
       </c>
       <c r="J21" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K21" s="2" t="inlineStr">
         <is>
@@ -1657,7 +1657,7 @@
         </is>
       </c>
       <c r="J22" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K22" s="2" t="inlineStr">
         <is>
@@ -1711,7 +1711,7 @@
         </is>
       </c>
       <c r="J23" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K23" s="2" t="inlineStr">
         <is>
@@ -1769,7 +1769,7 @@
         </is>
       </c>
       <c r="J24" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K24" s="2" t="inlineStr">
         <is>
@@ -1827,7 +1827,7 @@
         </is>
       </c>
       <c r="J25" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K25" s="2" t="inlineStr">
         <is>
@@ -1881,7 +1881,7 @@
         </is>
       </c>
       <c r="J26" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K26" s="2" t="inlineStr">
         <is>
@@ -1935,7 +1935,7 @@
         </is>
       </c>
       <c r="J27" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K27" s="2" t="inlineStr">
         <is>
@@ -1989,7 +1989,7 @@
         </is>
       </c>
       <c r="J28" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K28" s="2" t="inlineStr">
         <is>
@@ -2043,7 +2043,7 @@
         </is>
       </c>
       <c r="J29" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K29" s="2" t="inlineStr">
         <is>
@@ -2097,7 +2097,7 @@
         </is>
       </c>
       <c r="J30" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K30" s="2" t="inlineStr"/>
       <c r="L30" s="2" t="inlineStr">
@@ -2147,7 +2147,7 @@
         </is>
       </c>
       <c r="J31" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K31" s="2" t="inlineStr">
         <is>
@@ -2201,7 +2201,7 @@
         </is>
       </c>
       <c r="J32" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K32" s="2" t="inlineStr">
         <is>
@@ -2255,7 +2255,7 @@
         </is>
       </c>
       <c r="J33" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K33" s="2" t="inlineStr"/>
       <c r="L33" s="2" t="inlineStr">
@@ -2305,7 +2305,7 @@
         </is>
       </c>
       <c r="J34" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K34" s="2" t="inlineStr">
         <is>
@@ -2359,7 +2359,7 @@
         </is>
       </c>
       <c r="J35" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K35" s="2" t="inlineStr">
         <is>
@@ -2413,7 +2413,7 @@
         </is>
       </c>
       <c r="J36" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K36" s="2" t="inlineStr"/>
       <c r="L36" s="2" t="inlineStr">
@@ -2463,7 +2463,7 @@
         </is>
       </c>
       <c r="J37" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K37" s="2" t="inlineStr"/>
       <c r="L37" s="2" t="inlineStr">
@@ -2513,7 +2513,7 @@
         </is>
       </c>
       <c r="J38" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K38" s="2" t="inlineStr">
         <is>
@@ -2567,7 +2567,7 @@
         </is>
       </c>
       <c r="J39" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K39" s="2" t="inlineStr"/>
       <c r="L39" s="2" t="inlineStr">
@@ -2617,7 +2617,7 @@
         </is>
       </c>
       <c r="J40" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K40" s="2" t="inlineStr"/>
       <c r="L40" s="2" t="inlineStr">
@@ -2667,7 +2667,7 @@
         </is>
       </c>
       <c r="J41" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K41" s="2" t="inlineStr">
         <is>
@@ -2721,7 +2721,7 @@
         </is>
       </c>
       <c r="J42" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K42" s="2" t="inlineStr">
         <is>
@@ -2775,7 +2775,7 @@
         </is>
       </c>
       <c r="J43" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K43" s="2" t="inlineStr">
         <is>
@@ -2829,7 +2829,7 @@
         </is>
       </c>
       <c r="J44" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K44" s="2" t="inlineStr"/>
       <c r="L44" s="2" t="inlineStr">
@@ -2879,7 +2879,7 @@
         </is>
       </c>
       <c r="J45" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K45" s="2" t="inlineStr"/>
       <c r="L45" s="2" t="inlineStr">
@@ -2929,7 +2929,7 @@
         </is>
       </c>
       <c r="J46" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K46" s="2" t="inlineStr">
         <is>
@@ -2983,7 +2983,7 @@
         </is>
       </c>
       <c r="J47" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K47" s="2" t="inlineStr">
         <is>
@@ -3037,7 +3037,7 @@
         </is>
       </c>
       <c r="J48" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K48" s="2" t="inlineStr">
         <is>
@@ -3091,7 +3091,7 @@
         </is>
       </c>
       <c r="J49" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K49" s="2" t="inlineStr"/>
       <c r="L49" s="2" t="inlineStr">
@@ -3141,7 +3141,7 @@
         </is>
       </c>
       <c r="J50" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K50" s="2" t="inlineStr">
         <is>
@@ -3195,7 +3195,7 @@
         </is>
       </c>
       <c r="J51" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K51" s="2" t="inlineStr"/>
       <c r="L51" s="2" t="inlineStr">
@@ -3249,7 +3249,7 @@
         </is>
       </c>
       <c r="J52" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K52" s="2" t="inlineStr">
         <is>
@@ -3303,7 +3303,7 @@
         </is>
       </c>
       <c r="J53" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K53" s="2" t="inlineStr">
         <is>
@@ -3357,7 +3357,7 @@
         </is>
       </c>
       <c r="J54" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K54" s="2" t="inlineStr">
         <is>
@@ -3411,7 +3411,7 @@
         </is>
       </c>
       <c r="J55" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K55" s="2" t="inlineStr">
         <is>
@@ -3465,7 +3465,7 @@
         </is>
       </c>
       <c r="J56" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K56" s="2" t="inlineStr">
         <is>
@@ -3519,7 +3519,7 @@
         </is>
       </c>
       <c r="J57" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K57" s="2" t="inlineStr">
         <is>
@@ -3573,7 +3573,7 @@
         </is>
       </c>
       <c r="J58" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K58" s="2" t="inlineStr">
         <is>
@@ -3627,7 +3627,7 @@
         </is>
       </c>
       <c r="J59" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K59" s="2" t="inlineStr">
         <is>
@@ -3681,7 +3681,7 @@
         </is>
       </c>
       <c r="J60" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K60" s="2" t="inlineStr">
         <is>
@@ -3735,7 +3735,7 @@
         </is>
       </c>
       <c r="J61" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K61" s="2" t="inlineStr">
         <is>
@@ -3789,7 +3789,7 @@
         </is>
       </c>
       <c r="J62" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K62" s="2" t="inlineStr">
         <is>
@@ -3843,7 +3843,7 @@
         </is>
       </c>
       <c r="J63" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K63" s="2" t="inlineStr">
         <is>
@@ -3897,7 +3897,7 @@
         </is>
       </c>
       <c r="J64" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K64" s="2" t="inlineStr">
         <is>
@@ -3951,7 +3951,7 @@
         </is>
       </c>
       <c r="J65" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K65" s="2" t="inlineStr">
         <is>
@@ -4005,7 +4005,7 @@
         </is>
       </c>
       <c r="J66" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K66" s="2" t="inlineStr">
         <is>
@@ -4059,7 +4059,7 @@
         </is>
       </c>
       <c r="J67" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K67" s="2" t="inlineStr"/>
       <c r="L67" s="2" t="inlineStr">
@@ -4109,7 +4109,7 @@
         </is>
       </c>
       <c r="J68" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K68" s="2" t="inlineStr">
         <is>
@@ -4163,7 +4163,7 @@
         </is>
       </c>
       <c r="J69" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K69" s="2" t="inlineStr">
         <is>
@@ -4217,7 +4217,7 @@
         </is>
       </c>
       <c r="J70" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K70" s="2" t="inlineStr">
         <is>
@@ -4271,7 +4271,7 @@
         </is>
       </c>
       <c r="J71" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K71" s="2" t="inlineStr"/>
       <c r="L71" s="2" t="inlineStr">
@@ -4321,7 +4321,7 @@
         </is>
       </c>
       <c r="J72" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K72" s="2" t="inlineStr"/>
       <c r="L72" s="2" t="inlineStr">
@@ -4371,7 +4371,7 @@
         </is>
       </c>
       <c r="J73" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K73" s="2" t="inlineStr">
         <is>
@@ -4425,7 +4425,7 @@
         </is>
       </c>
       <c r="J74" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K74" s="2" t="inlineStr">
         <is>
@@ -4479,7 +4479,7 @@
         </is>
       </c>
       <c r="J75" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K75" s="2" t="inlineStr">
         <is>
@@ -4533,7 +4533,7 @@
         </is>
       </c>
       <c r="J76" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K76" s="2" t="inlineStr"/>
       <c r="L76" s="2" t="inlineStr">
@@ -4583,7 +4583,7 @@
         </is>
       </c>
       <c r="J77" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K77" s="2" t="inlineStr"/>
       <c r="L77" s="2" t="inlineStr">
@@ -4633,7 +4633,7 @@
         </is>
       </c>
       <c r="J78" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K78" s="2" t="inlineStr"/>
       <c r="L78" s="2" t="inlineStr">
@@ -4683,7 +4683,7 @@
         </is>
       </c>
       <c r="J79" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K79" s="2" t="inlineStr">
         <is>
@@ -4737,7 +4737,7 @@
         </is>
       </c>
       <c r="J80" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K80" s="2" t="inlineStr"/>
       <c r="L80" s="2" t="inlineStr">
@@ -4787,7 +4787,7 @@
         </is>
       </c>
       <c r="J81" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K81" s="2" t="inlineStr">
         <is>
@@ -4845,7 +4845,7 @@
         </is>
       </c>
       <c r="J82" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K82" s="2" t="inlineStr">
         <is>
@@ -4903,7 +4903,7 @@
         </is>
       </c>
       <c r="J83" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K83" s="2" t="inlineStr">
         <is>
@@ -4957,7 +4957,7 @@
         </is>
       </c>
       <c r="J84" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K84" s="2" t="inlineStr">
         <is>
@@ -5011,7 +5011,7 @@
         </is>
       </c>
       <c r="J85" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K85" s="2" t="inlineStr">
         <is>
@@ -5065,7 +5065,7 @@
         </is>
       </c>
       <c r="J86" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K86" s="2" t="inlineStr">
         <is>
@@ -5119,7 +5119,7 @@
         </is>
       </c>
       <c r="J87" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K87" s="2" t="inlineStr">
         <is>
@@ -5173,7 +5173,7 @@
         </is>
       </c>
       <c r="J88" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K88" s="2" t="inlineStr"/>
       <c r="L88" s="2" t="inlineStr">
@@ -5223,7 +5223,7 @@
         </is>
       </c>
       <c r="J89" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K89" s="2" t="inlineStr">
         <is>
@@ -5277,7 +5277,7 @@
         </is>
       </c>
       <c r="J90" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K90" s="2" t="inlineStr">
         <is>
@@ -5331,7 +5331,7 @@
         </is>
       </c>
       <c r="J91" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K91" s="2" t="inlineStr">
         <is>
@@ -5385,7 +5385,7 @@
         </is>
       </c>
       <c r="J92" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K92" s="2" t="inlineStr"/>
       <c r="L92" s="2" t="inlineStr">
@@ -5435,7 +5435,7 @@
         </is>
       </c>
       <c r="J93" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K93" s="2" t="inlineStr">
         <is>
@@ -5489,7 +5489,7 @@
         </is>
       </c>
       <c r="J94" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K94" s="2" t="inlineStr">
         <is>
@@ -5543,7 +5543,7 @@
         </is>
       </c>
       <c r="J95" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K95" s="2" t="inlineStr">
         <is>
@@ -5597,7 +5597,7 @@
         </is>
       </c>
       <c r="J96" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K96" s="2" t="inlineStr"/>
       <c r="L96" s="2" t="inlineStr">
@@ -5647,7 +5647,7 @@
         </is>
       </c>
       <c r="J97" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K97" s="2" t="inlineStr"/>
       <c r="L97" s="2" t="inlineStr">
@@ -5697,7 +5697,7 @@
         </is>
       </c>
       <c r="J98" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K98" s="2" t="inlineStr">
         <is>
@@ -5751,7 +5751,7 @@
         </is>
       </c>
       <c r="J99" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K99" s="2" t="inlineStr">
         <is>
@@ -5805,7 +5805,7 @@
         </is>
       </c>
       <c r="J100" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K100" s="2" t="inlineStr"/>
       <c r="L100" s="2" t="inlineStr">
@@ -5855,7 +5855,7 @@
         </is>
       </c>
       <c r="J101" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K101" s="2" t="inlineStr">
         <is>
@@ -5909,7 +5909,7 @@
         </is>
       </c>
       <c r="J102" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K102" s="2" t="inlineStr">
         <is>
@@ -5963,7 +5963,7 @@
         </is>
       </c>
       <c r="J103" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K103" s="2" t="inlineStr">
         <is>
@@ -6017,7 +6017,7 @@
         </is>
       </c>
       <c r="J104" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K104" s="2" t="inlineStr">
         <is>
@@ -6071,7 +6071,7 @@
         </is>
       </c>
       <c r="J105" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K105" s="2" t="inlineStr"/>
       <c r="L105" s="2" t="inlineStr">
@@ -6121,7 +6121,7 @@
         </is>
       </c>
       <c r="J106" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K106" s="2" t="inlineStr">
         <is>
@@ -6175,7 +6175,7 @@
         </is>
       </c>
       <c r="J107" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K107" s="2" t="inlineStr">
         <is>
@@ -6229,7 +6229,7 @@
         </is>
       </c>
       <c r="J108" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K108" s="2" t="inlineStr">
         <is>
@@ -6283,7 +6283,7 @@
         </is>
       </c>
       <c r="J109" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K109" s="2" t="inlineStr"/>
       <c r="L109" s="2" t="inlineStr">
@@ -6333,7 +6333,7 @@
         </is>
       </c>
       <c r="J110" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K110" s="2" t="inlineStr"/>
       <c r="L110" s="2" t="inlineStr">
@@ -6383,7 +6383,7 @@
         </is>
       </c>
       <c r="J111" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K111" s="2" t="inlineStr">
         <is>
@@ -6437,7 +6437,7 @@
         </is>
       </c>
       <c r="J112" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K112" s="2" t="inlineStr">
         <is>
@@ -6491,7 +6491,7 @@
         </is>
       </c>
       <c r="J113" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K113" s="2" t="inlineStr">
         <is>
@@ -7188,7 +7188,7 @@
         </is>
       </c>
       <c r="C2" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="3">
@@ -7203,7 +7203,7 @@
         </is>
       </c>
       <c r="C3" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="4">
@@ -7218,7 +7218,7 @@
         </is>
       </c>
       <c r="C4" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="5">
@@ -7233,7 +7233,7 @@
         </is>
       </c>
       <c r="C5" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="6">
@@ -7248,7 +7248,7 @@
         </is>
       </c>
       <c r="C6" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="7">
@@ -7263,7 +7263,7 @@
         </is>
       </c>
       <c r="C7" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="8">
@@ -7278,7 +7278,7 @@
         </is>
       </c>
       <c r="C8" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="9">
@@ -7293,7 +7293,7 @@
         </is>
       </c>
       <c r="C9" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="10">
@@ -7308,7 +7308,7 @@
         </is>
       </c>
       <c r="C10" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="11">
@@ -7323,7 +7323,7 @@
         </is>
       </c>
       <c r="C11" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="12">
@@ -7338,7 +7338,7 @@
         </is>
       </c>
       <c r="C12" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="13">
@@ -7353,7 +7353,7 @@
         </is>
       </c>
       <c r="C13" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="14">
@@ -7368,7 +7368,7 @@
         </is>
       </c>
       <c r="C14" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="15">
@@ -7383,7 +7383,7 @@
         </is>
       </c>
       <c r="C15" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="16">
@@ -7398,7 +7398,7 @@
         </is>
       </c>
       <c r="C16" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="17">
@@ -7413,7 +7413,7 @@
         </is>
       </c>
       <c r="C17" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="18">
@@ -7428,7 +7428,7 @@
         </is>
       </c>
       <c r="C18" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="19">
@@ -7443,7 +7443,7 @@
         </is>
       </c>
       <c r="C19" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="20">
@@ -7458,7 +7458,7 @@
         </is>
       </c>
       <c r="C20" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="21">
@@ -7473,7 +7473,7 @@
         </is>
       </c>
       <c r="C21" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="22">
@@ -7488,7 +7488,7 @@
         </is>
       </c>
       <c r="C22" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="23">
@@ -7503,7 +7503,7 @@
         </is>
       </c>
       <c r="C23" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="24">
@@ -7518,7 +7518,7 @@
         </is>
       </c>
       <c r="C24" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="25">
@@ -7533,7 +7533,7 @@
         </is>
       </c>
       <c r="C25" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="26">
@@ -7548,7 +7548,7 @@
         </is>
       </c>
       <c r="C26" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="27">
@@ -7563,7 +7563,7 @@
         </is>
       </c>
       <c r="C27" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="28">
@@ -7578,7 +7578,7 @@
         </is>
       </c>
       <c r="C28" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="29">
@@ -7593,7 +7593,7 @@
         </is>
       </c>
       <c r="C29" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="30">
@@ -7608,7 +7608,7 @@
         </is>
       </c>
       <c r="C30" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="31">
@@ -7623,7 +7623,7 @@
         </is>
       </c>
       <c r="C31" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="32">
@@ -7638,7 +7638,7 @@
         </is>
       </c>
       <c r="C32" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="33">
@@ -7653,7 +7653,7 @@
         </is>
       </c>
       <c r="C33" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="34">
@@ -7668,7 +7668,7 @@
         </is>
       </c>
       <c r="C34" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="35">
@@ -7683,7 +7683,7 @@
         </is>
       </c>
       <c r="C35" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="36">
@@ -7698,7 +7698,7 @@
         </is>
       </c>
       <c r="C36" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="37">
@@ -7713,7 +7713,7 @@
         </is>
       </c>
       <c r="C37" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="38">
@@ -7728,7 +7728,7 @@
         </is>
       </c>
       <c r="C38" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="39">
@@ -7743,7 +7743,7 @@
         </is>
       </c>
       <c r="C39" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="40">
@@ -7758,7 +7758,7 @@
         </is>
       </c>
       <c r="C40" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="41">
@@ -7773,7 +7773,7 @@
         </is>
       </c>
       <c r="C41" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="42">
@@ -7788,7 +7788,7 @@
         </is>
       </c>
       <c r="C42" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="43">
@@ -7803,7 +7803,7 @@
         </is>
       </c>
       <c r="C43" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="44">
@@ -7818,7 +7818,7 @@
         </is>
       </c>
       <c r="C44" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="45">
@@ -7833,7 +7833,7 @@
         </is>
       </c>
       <c r="C45" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="46">
@@ -7848,7 +7848,7 @@
         </is>
       </c>
       <c r="C46" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="47">
@@ -7863,7 +7863,7 @@
         </is>
       </c>
       <c r="C47" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="48">
@@ -7878,7 +7878,7 @@
         </is>
       </c>
       <c r="C48" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="49">
@@ -7893,7 +7893,7 @@
         </is>
       </c>
       <c r="C49" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="50">
@@ -7908,7 +7908,7 @@
         </is>
       </c>
       <c r="C50" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="51">
@@ -7923,7 +7923,7 @@
         </is>
       </c>
       <c r="C51" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="52">
@@ -7938,7 +7938,7 @@
         </is>
       </c>
       <c r="C52" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="53">
@@ -7953,7 +7953,7 @@
         </is>
       </c>
       <c r="C53" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="54">
@@ -7968,7 +7968,7 @@
         </is>
       </c>
       <c r="C54" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="55">
@@ -7983,7 +7983,7 @@
         </is>
       </c>
       <c r="C55" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="56">
@@ -7998,7 +7998,7 @@
         </is>
       </c>
       <c r="C56" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="57">
@@ -8013,7 +8013,7 @@
         </is>
       </c>
       <c r="C57" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="58">
@@ -8028,7 +8028,7 @@
         </is>
       </c>
       <c r="C58" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="59">
@@ -8043,7 +8043,7 @@
         </is>
       </c>
       <c r="C59" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="60">
@@ -8058,7 +8058,7 @@
         </is>
       </c>
       <c r="C60" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="61">
@@ -8073,7 +8073,7 @@
         </is>
       </c>
       <c r="C61" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="62">
@@ -8088,7 +8088,7 @@
         </is>
       </c>
       <c r="C62" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="63">
@@ -8103,7 +8103,7 @@
         </is>
       </c>
       <c r="C63" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="64">
@@ -8118,7 +8118,7 @@
         </is>
       </c>
       <c r="C64" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="65">
@@ -8133,7 +8133,7 @@
         </is>
       </c>
       <c r="C65" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="66">
@@ -8148,7 +8148,7 @@
         </is>
       </c>
       <c r="C66" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="67">
@@ -8163,7 +8163,7 @@
         </is>
       </c>
       <c r="C67" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="68">
@@ -8178,7 +8178,7 @@
         </is>
       </c>
       <c r="C68" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="69">
@@ -8193,7 +8193,7 @@
         </is>
       </c>
       <c r="C69" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="70">
@@ -8208,7 +8208,7 @@
         </is>
       </c>
       <c r="C70" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="71">
@@ -8223,7 +8223,7 @@
         </is>
       </c>
       <c r="C71" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="72">
@@ -8238,7 +8238,7 @@
         </is>
       </c>
       <c r="C72" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="73">
@@ -8253,7 +8253,7 @@
         </is>
       </c>
       <c r="C73" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="74">
@@ -8268,7 +8268,7 @@
         </is>
       </c>
       <c r="C74" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="75">
@@ -8283,7 +8283,7 @@
         </is>
       </c>
       <c r="C75" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="76">
@@ -8298,7 +8298,7 @@
         </is>
       </c>
       <c r="C76" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="77">
@@ -8313,7 +8313,7 @@
         </is>
       </c>
       <c r="C77" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="78">
@@ -8328,7 +8328,7 @@
         </is>
       </c>
       <c r="C78" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="79">
@@ -8343,7 +8343,7 @@
         </is>
       </c>
       <c r="C79" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="80">
@@ -8358,7 +8358,7 @@
         </is>
       </c>
       <c r="C80" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="81">
@@ -8373,7 +8373,7 @@
         </is>
       </c>
       <c r="C81" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="82">
@@ -8388,7 +8388,7 @@
         </is>
       </c>
       <c r="C82" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="83">
@@ -8403,7 +8403,7 @@
         </is>
       </c>
       <c r="C83" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="84">
@@ -8418,7 +8418,7 @@
         </is>
       </c>
       <c r="C84" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="85">
@@ -8433,7 +8433,7 @@
         </is>
       </c>
       <c r="C85" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="86">
@@ -8448,7 +8448,7 @@
         </is>
       </c>
       <c r="C86" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="87">
@@ -8463,7 +8463,7 @@
         </is>
       </c>
       <c r="C87" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="88">
@@ -8478,7 +8478,7 @@
         </is>
       </c>
       <c r="C88" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="89">
@@ -8493,7 +8493,7 @@
         </is>
       </c>
       <c r="C89" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="90">
@@ -8508,7 +8508,7 @@
         </is>
       </c>
       <c r="C90" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="91">
@@ -8523,7 +8523,7 @@
         </is>
       </c>
       <c r="C91" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="92">
@@ -8538,7 +8538,7 @@
         </is>
       </c>
       <c r="C92" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="93">
@@ -8553,7 +8553,7 @@
         </is>
       </c>
       <c r="C93" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="94">
@@ -8568,7 +8568,7 @@
         </is>
       </c>
       <c r="C94" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="95">
@@ -8583,7 +8583,7 @@
         </is>
       </c>
       <c r="C95" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="96">
@@ -8598,7 +8598,7 @@
         </is>
       </c>
       <c r="C96" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="97">
@@ -8613,7 +8613,7 @@
         </is>
       </c>
       <c r="C97" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="98">
@@ -8628,7 +8628,7 @@
         </is>
       </c>
       <c r="C98" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="99">
@@ -8643,7 +8643,7 @@
         </is>
       </c>
       <c r="C99" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="100">
@@ -8658,7 +8658,7 @@
         </is>
       </c>
       <c r="C100" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="101">
@@ -8673,7 +8673,7 @@
         </is>
       </c>
       <c r="C101" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="102">
@@ -8688,7 +8688,7 @@
         </is>
       </c>
       <c r="C102" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="103">
@@ -8703,7 +8703,7 @@
         </is>
       </c>
       <c r="C103" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="104">
@@ -8718,7 +8718,7 @@
         </is>
       </c>
       <c r="C104" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="105">
@@ -8733,7 +8733,7 @@
         </is>
       </c>
       <c r="C105" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="106">
@@ -8748,7 +8748,7 @@
         </is>
       </c>
       <c r="C106" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="107">
@@ -8763,7 +8763,7 @@
         </is>
       </c>
       <c r="C107" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="108">
@@ -8778,7 +8778,7 @@
         </is>
       </c>
       <c r="C108" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="109">
@@ -8793,7 +8793,7 @@
         </is>
       </c>
       <c r="C109" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="110">
@@ -8808,7 +8808,7 @@
         </is>
       </c>
       <c r="C110" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="111">
@@ -8823,7 +8823,7 @@
         </is>
       </c>
       <c r="C111" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="112">
@@ -8838,7 +8838,7 @@
         </is>
       </c>
       <c r="C112" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="113">
@@ -8853,7 +8853,7 @@
         </is>
       </c>
       <c r="C113" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
radar 2026-09-05: +0 novas, 0 atualizadas, 0 snapshots
</commit_message>
<xml_diff>
--- a/Radar/radar-low-ticket.xlsx
+++ b/Radar/radar-low-ticket.xlsx
@@ -565,7 +565,7 @@
         </is>
       </c>
       <c r="J2" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K2" s="2" t="inlineStr">
         <is>
@@ -619,7 +619,7 @@
         </is>
       </c>
       <c r="J3" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
@@ -673,7 +673,7 @@
         </is>
       </c>
       <c r="J4" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K4" s="2" t="inlineStr">
         <is>
@@ -727,7 +727,7 @@
         </is>
       </c>
       <c r="J5" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K5" s="2" t="inlineStr">
         <is>
@@ -785,7 +785,7 @@
         </is>
       </c>
       <c r="J6" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K6" s="2" t="inlineStr">
         <is>
@@ -839,7 +839,7 @@
         </is>
       </c>
       <c r="J7" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K7" s="2" t="inlineStr"/>
       <c r="L7" s="2" t="inlineStr">
@@ -893,7 +893,7 @@
         </is>
       </c>
       <c r="J8" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K8" s="2" t="inlineStr">
         <is>
@@ -947,7 +947,7 @@
         </is>
       </c>
       <c r="J9" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K9" s="2" t="inlineStr"/>
       <c r="L9" s="2" t="inlineStr">
@@ -997,7 +997,7 @@
         </is>
       </c>
       <c r="J10" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K10" s="2" t="inlineStr">
         <is>
@@ -1055,7 +1055,7 @@
         </is>
       </c>
       <c r="J11" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K11" s="2" t="inlineStr">
         <is>
@@ -1109,7 +1109,7 @@
         </is>
       </c>
       <c r="J12" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K12" s="2" t="inlineStr">
         <is>
@@ -1167,7 +1167,7 @@
         </is>
       </c>
       <c r="J13" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K13" s="2" t="inlineStr">
         <is>
@@ -1221,7 +1221,7 @@
         </is>
       </c>
       <c r="J14" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K14" s="2" t="inlineStr">
         <is>
@@ -1275,7 +1275,7 @@
         </is>
       </c>
       <c r="J15" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K15" s="2" t="inlineStr">
         <is>
@@ -1329,7 +1329,7 @@
         </is>
       </c>
       <c r="J16" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K16" s="2" t="inlineStr">
         <is>
@@ -1387,7 +1387,7 @@
         </is>
       </c>
       <c r="J17" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K17" s="2" t="inlineStr"/>
       <c r="L17" s="2" t="inlineStr">
@@ -1437,7 +1437,7 @@
         </is>
       </c>
       <c r="J18" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K18" s="2" t="inlineStr">
         <is>
@@ -1491,7 +1491,7 @@
         </is>
       </c>
       <c r="J19" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K19" s="2" t="inlineStr">
         <is>
@@ -1545,7 +1545,7 @@
         </is>
       </c>
       <c r="J20" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K20" s="2" t="inlineStr">
         <is>
@@ -1599,7 +1599,7 @@
         </is>
       </c>
       <c r="J21" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K21" s="2" t="inlineStr">
         <is>
@@ -1657,7 +1657,7 @@
         </is>
       </c>
       <c r="J22" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K22" s="2" t="inlineStr">
         <is>
@@ -1711,7 +1711,7 @@
         </is>
       </c>
       <c r="J23" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K23" s="2" t="inlineStr">
         <is>
@@ -1769,7 +1769,7 @@
         </is>
       </c>
       <c r="J24" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K24" s="2" t="inlineStr">
         <is>
@@ -1827,7 +1827,7 @@
         </is>
       </c>
       <c r="J25" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K25" s="2" t="inlineStr">
         <is>
@@ -1881,7 +1881,7 @@
         </is>
       </c>
       <c r="J26" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K26" s="2" t="inlineStr">
         <is>
@@ -1935,7 +1935,7 @@
         </is>
       </c>
       <c r="J27" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K27" s="2" t="inlineStr">
         <is>
@@ -1989,7 +1989,7 @@
         </is>
       </c>
       <c r="J28" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K28" s="2" t="inlineStr">
         <is>
@@ -2043,7 +2043,7 @@
         </is>
       </c>
       <c r="J29" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K29" s="2" t="inlineStr">
         <is>
@@ -2097,7 +2097,7 @@
         </is>
       </c>
       <c r="J30" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K30" s="2" t="inlineStr"/>
       <c r="L30" s="2" t="inlineStr">
@@ -2147,7 +2147,7 @@
         </is>
       </c>
       <c r="J31" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K31" s="2" t="inlineStr">
         <is>
@@ -2201,7 +2201,7 @@
         </is>
       </c>
       <c r="J32" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K32" s="2" t="inlineStr">
         <is>
@@ -2255,7 +2255,7 @@
         </is>
       </c>
       <c r="J33" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K33" s="2" t="inlineStr"/>
       <c r="L33" s="2" t="inlineStr">
@@ -2305,7 +2305,7 @@
         </is>
       </c>
       <c r="J34" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K34" s="2" t="inlineStr">
         <is>
@@ -2359,7 +2359,7 @@
         </is>
       </c>
       <c r="J35" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K35" s="2" t="inlineStr">
         <is>
@@ -2413,7 +2413,7 @@
         </is>
       </c>
       <c r="J36" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K36" s="2" t="inlineStr"/>
       <c r="L36" s="2" t="inlineStr">
@@ -2463,7 +2463,7 @@
         </is>
       </c>
       <c r="J37" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K37" s="2" t="inlineStr"/>
       <c r="L37" s="2" t="inlineStr">
@@ -2513,7 +2513,7 @@
         </is>
       </c>
       <c r="J38" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K38" s="2" t="inlineStr">
         <is>
@@ -2567,7 +2567,7 @@
         </is>
       </c>
       <c r="J39" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K39" s="2" t="inlineStr"/>
       <c r="L39" s="2" t="inlineStr">
@@ -2617,7 +2617,7 @@
         </is>
       </c>
       <c r="J40" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K40" s="2" t="inlineStr"/>
       <c r="L40" s="2" t="inlineStr">
@@ -2667,7 +2667,7 @@
         </is>
       </c>
       <c r="J41" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K41" s="2" t="inlineStr">
         <is>
@@ -2721,7 +2721,7 @@
         </is>
       </c>
       <c r="J42" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K42" s="2" t="inlineStr">
         <is>
@@ -2775,7 +2775,7 @@
         </is>
       </c>
       <c r="J43" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K43" s="2" t="inlineStr">
         <is>
@@ -2829,7 +2829,7 @@
         </is>
       </c>
       <c r="J44" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K44" s="2" t="inlineStr"/>
       <c r="L44" s="2" t="inlineStr">
@@ -2879,7 +2879,7 @@
         </is>
       </c>
       <c r="J45" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K45" s="2" t="inlineStr"/>
       <c r="L45" s="2" t="inlineStr">
@@ -2929,7 +2929,7 @@
         </is>
       </c>
       <c r="J46" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K46" s="2" t="inlineStr">
         <is>
@@ -2983,7 +2983,7 @@
         </is>
       </c>
       <c r="J47" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K47" s="2" t="inlineStr">
         <is>
@@ -3037,7 +3037,7 @@
         </is>
       </c>
       <c r="J48" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K48" s="2" t="inlineStr">
         <is>
@@ -3091,7 +3091,7 @@
         </is>
       </c>
       <c r="J49" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K49" s="2" t="inlineStr"/>
       <c r="L49" s="2" t="inlineStr">
@@ -3141,7 +3141,7 @@
         </is>
       </c>
       <c r="J50" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K50" s="2" t="inlineStr">
         <is>
@@ -3195,7 +3195,7 @@
         </is>
       </c>
       <c r="J51" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K51" s="2" t="inlineStr"/>
       <c r="L51" s="2" t="inlineStr">
@@ -3249,7 +3249,7 @@
         </is>
       </c>
       <c r="J52" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K52" s="2" t="inlineStr">
         <is>
@@ -3303,7 +3303,7 @@
         </is>
       </c>
       <c r="J53" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K53" s="2" t="inlineStr">
         <is>
@@ -3357,7 +3357,7 @@
         </is>
       </c>
       <c r="J54" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K54" s="2" t="inlineStr">
         <is>
@@ -3411,7 +3411,7 @@
         </is>
       </c>
       <c r="J55" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K55" s="2" t="inlineStr">
         <is>
@@ -3465,7 +3465,7 @@
         </is>
       </c>
       <c r="J56" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K56" s="2" t="inlineStr">
         <is>
@@ -3519,7 +3519,7 @@
         </is>
       </c>
       <c r="J57" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K57" s="2" t="inlineStr">
         <is>
@@ -3573,7 +3573,7 @@
         </is>
       </c>
       <c r="J58" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K58" s="2" t="inlineStr">
         <is>
@@ -3627,7 +3627,7 @@
         </is>
       </c>
       <c r="J59" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K59" s="2" t="inlineStr">
         <is>
@@ -3681,7 +3681,7 @@
         </is>
       </c>
       <c r="J60" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K60" s="2" t="inlineStr">
         <is>
@@ -3735,7 +3735,7 @@
         </is>
       </c>
       <c r="J61" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K61" s="2" t="inlineStr">
         <is>
@@ -3789,7 +3789,7 @@
         </is>
       </c>
       <c r="J62" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K62" s="2" t="inlineStr">
         <is>
@@ -3843,7 +3843,7 @@
         </is>
       </c>
       <c r="J63" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K63" s="2" t="inlineStr">
         <is>
@@ -3897,7 +3897,7 @@
         </is>
       </c>
       <c r="J64" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K64" s="2" t="inlineStr">
         <is>
@@ -3951,7 +3951,7 @@
         </is>
       </c>
       <c r="J65" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K65" s="2" t="inlineStr">
         <is>
@@ -4005,7 +4005,7 @@
         </is>
       </c>
       <c r="J66" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K66" s="2" t="inlineStr">
         <is>
@@ -4059,7 +4059,7 @@
         </is>
       </c>
       <c r="J67" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K67" s="2" t="inlineStr"/>
       <c r="L67" s="2" t="inlineStr">
@@ -4109,7 +4109,7 @@
         </is>
       </c>
       <c r="J68" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K68" s="2" t="inlineStr">
         <is>
@@ -4163,7 +4163,7 @@
         </is>
       </c>
       <c r="J69" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K69" s="2" t="inlineStr">
         <is>
@@ -4217,7 +4217,7 @@
         </is>
       </c>
       <c r="J70" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K70" s="2" t="inlineStr">
         <is>
@@ -4271,7 +4271,7 @@
         </is>
       </c>
       <c r="J71" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K71" s="2" t="inlineStr"/>
       <c r="L71" s="2" t="inlineStr">
@@ -4321,7 +4321,7 @@
         </is>
       </c>
       <c r="J72" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K72" s="2" t="inlineStr"/>
       <c r="L72" s="2" t="inlineStr">
@@ -4371,7 +4371,7 @@
         </is>
       </c>
       <c r="J73" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K73" s="2" t="inlineStr">
         <is>
@@ -4425,7 +4425,7 @@
         </is>
       </c>
       <c r="J74" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K74" s="2" t="inlineStr">
         <is>
@@ -4479,7 +4479,7 @@
         </is>
       </c>
       <c r="J75" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K75" s="2" t="inlineStr">
         <is>
@@ -4533,7 +4533,7 @@
         </is>
       </c>
       <c r="J76" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K76" s="2" t="inlineStr"/>
       <c r="L76" s="2" t="inlineStr">
@@ -4583,7 +4583,7 @@
         </is>
       </c>
       <c r="J77" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K77" s="2" t="inlineStr"/>
       <c r="L77" s="2" t="inlineStr">
@@ -4633,7 +4633,7 @@
         </is>
       </c>
       <c r="J78" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K78" s="2" t="inlineStr"/>
       <c r="L78" s="2" t="inlineStr">
@@ -4683,7 +4683,7 @@
         </is>
       </c>
       <c r="J79" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K79" s="2" t="inlineStr">
         <is>
@@ -4737,7 +4737,7 @@
         </is>
       </c>
       <c r="J80" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K80" s="2" t="inlineStr"/>
       <c r="L80" s="2" t="inlineStr">
@@ -4787,7 +4787,7 @@
         </is>
       </c>
       <c r="J81" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K81" s="2" t="inlineStr">
         <is>
@@ -4845,7 +4845,7 @@
         </is>
       </c>
       <c r="J82" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K82" s="2" t="inlineStr">
         <is>
@@ -4903,7 +4903,7 @@
         </is>
       </c>
       <c r="J83" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K83" s="2" t="inlineStr">
         <is>
@@ -4957,7 +4957,7 @@
         </is>
       </c>
       <c r="J84" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K84" s="2" t="inlineStr">
         <is>
@@ -5011,7 +5011,7 @@
         </is>
       </c>
       <c r="J85" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K85" s="2" t="inlineStr">
         <is>
@@ -5065,7 +5065,7 @@
         </is>
       </c>
       <c r="J86" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K86" s="2" t="inlineStr">
         <is>
@@ -5119,7 +5119,7 @@
         </is>
       </c>
       <c r="J87" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K87" s="2" t="inlineStr">
         <is>
@@ -5173,7 +5173,7 @@
         </is>
       </c>
       <c r="J88" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K88" s="2" t="inlineStr"/>
       <c r="L88" s="2" t="inlineStr">
@@ -5223,7 +5223,7 @@
         </is>
       </c>
       <c r="J89" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K89" s="2" t="inlineStr">
         <is>
@@ -5277,7 +5277,7 @@
         </is>
       </c>
       <c r="J90" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K90" s="2" t="inlineStr">
         <is>
@@ -5331,7 +5331,7 @@
         </is>
       </c>
       <c r="J91" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K91" s="2" t="inlineStr">
         <is>
@@ -5385,7 +5385,7 @@
         </is>
       </c>
       <c r="J92" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K92" s="2" t="inlineStr"/>
       <c r="L92" s="2" t="inlineStr">
@@ -5435,7 +5435,7 @@
         </is>
       </c>
       <c r="J93" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K93" s="2" t="inlineStr">
         <is>
@@ -5489,7 +5489,7 @@
         </is>
       </c>
       <c r="J94" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K94" s="2" t="inlineStr">
         <is>
@@ -5543,7 +5543,7 @@
         </is>
       </c>
       <c r="J95" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K95" s="2" t="inlineStr">
         <is>
@@ -5597,7 +5597,7 @@
         </is>
       </c>
       <c r="J96" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K96" s="2" t="inlineStr"/>
       <c r="L96" s="2" t="inlineStr">
@@ -5647,7 +5647,7 @@
         </is>
       </c>
       <c r="J97" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K97" s="2" t="inlineStr"/>
       <c r="L97" s="2" t="inlineStr">
@@ -5697,7 +5697,7 @@
         </is>
       </c>
       <c r="J98" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K98" s="2" t="inlineStr">
         <is>
@@ -5751,7 +5751,7 @@
         </is>
       </c>
       <c r="J99" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K99" s="2" t="inlineStr">
         <is>
@@ -5805,7 +5805,7 @@
         </is>
       </c>
       <c r="J100" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K100" s="2" t="inlineStr"/>
       <c r="L100" s="2" t="inlineStr">
@@ -5855,7 +5855,7 @@
         </is>
       </c>
       <c r="J101" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K101" s="2" t="inlineStr">
         <is>
@@ -5909,7 +5909,7 @@
         </is>
       </c>
       <c r="J102" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K102" s="2" t="inlineStr">
         <is>
@@ -5963,7 +5963,7 @@
         </is>
       </c>
       <c r="J103" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K103" s="2" t="inlineStr">
         <is>
@@ -6017,7 +6017,7 @@
         </is>
       </c>
       <c r="J104" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K104" s="2" t="inlineStr">
         <is>
@@ -6071,7 +6071,7 @@
         </is>
       </c>
       <c r="J105" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K105" s="2" t="inlineStr"/>
       <c r="L105" s="2" t="inlineStr">
@@ -6121,7 +6121,7 @@
         </is>
       </c>
       <c r="J106" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K106" s="2" t="inlineStr">
         <is>
@@ -6175,7 +6175,7 @@
         </is>
       </c>
       <c r="J107" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K107" s="2" t="inlineStr">
         <is>
@@ -6229,7 +6229,7 @@
         </is>
       </c>
       <c r="J108" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K108" s="2" t="inlineStr">
         <is>
@@ -6283,7 +6283,7 @@
         </is>
       </c>
       <c r="J109" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K109" s="2" t="inlineStr"/>
       <c r="L109" s="2" t="inlineStr">
@@ -6333,7 +6333,7 @@
         </is>
       </c>
       <c r="J110" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K110" s="2" t="inlineStr"/>
       <c r="L110" s="2" t="inlineStr">
@@ -6383,7 +6383,7 @@
         </is>
       </c>
       <c r="J111" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K111" s="2" t="inlineStr">
         <is>
@@ -6437,7 +6437,7 @@
         </is>
       </c>
       <c r="J112" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K112" s="2" t="inlineStr">
         <is>
@@ -6491,7 +6491,7 @@
         </is>
       </c>
       <c r="J113" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K113" s="2" t="inlineStr">
         <is>
@@ -7188,7 +7188,7 @@
         </is>
       </c>
       <c r="C2" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="3">
@@ -7203,7 +7203,7 @@
         </is>
       </c>
       <c r="C3" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="4">
@@ -7218,7 +7218,7 @@
         </is>
       </c>
       <c r="C4" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="5">
@@ -7233,7 +7233,7 @@
         </is>
       </c>
       <c r="C5" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="6">
@@ -7248,7 +7248,7 @@
         </is>
       </c>
       <c r="C6" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="7">
@@ -7263,7 +7263,7 @@
         </is>
       </c>
       <c r="C7" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="8">
@@ -7278,7 +7278,7 @@
         </is>
       </c>
       <c r="C8" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="9">
@@ -7293,7 +7293,7 @@
         </is>
       </c>
       <c r="C9" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="10">
@@ -7308,7 +7308,7 @@
         </is>
       </c>
       <c r="C10" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="11">
@@ -7323,7 +7323,7 @@
         </is>
       </c>
       <c r="C11" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="12">
@@ -7338,7 +7338,7 @@
         </is>
       </c>
       <c r="C12" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="13">
@@ -7353,7 +7353,7 @@
         </is>
       </c>
       <c r="C13" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="14">
@@ -7368,7 +7368,7 @@
         </is>
       </c>
       <c r="C14" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="15">
@@ -7383,7 +7383,7 @@
         </is>
       </c>
       <c r="C15" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="16">
@@ -7398,7 +7398,7 @@
         </is>
       </c>
       <c r="C16" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="17">
@@ -7413,7 +7413,7 @@
         </is>
       </c>
       <c r="C17" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="18">
@@ -7428,7 +7428,7 @@
         </is>
       </c>
       <c r="C18" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="19">
@@ -7443,7 +7443,7 @@
         </is>
       </c>
       <c r="C19" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="20">
@@ -7458,7 +7458,7 @@
         </is>
       </c>
       <c r="C20" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="21">
@@ -7473,7 +7473,7 @@
         </is>
       </c>
       <c r="C21" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="22">
@@ -7488,7 +7488,7 @@
         </is>
       </c>
       <c r="C22" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="23">
@@ -7503,7 +7503,7 @@
         </is>
       </c>
       <c r="C23" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="24">
@@ -7518,7 +7518,7 @@
         </is>
       </c>
       <c r="C24" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="25">
@@ -7533,7 +7533,7 @@
         </is>
       </c>
       <c r="C25" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="26">
@@ -7548,7 +7548,7 @@
         </is>
       </c>
       <c r="C26" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="27">
@@ -7563,7 +7563,7 @@
         </is>
       </c>
       <c r="C27" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="28">
@@ -7578,7 +7578,7 @@
         </is>
       </c>
       <c r="C28" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="29">
@@ -7593,7 +7593,7 @@
         </is>
       </c>
       <c r="C29" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="30">
@@ -7608,7 +7608,7 @@
         </is>
       </c>
       <c r="C30" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="31">
@@ -7623,7 +7623,7 @@
         </is>
       </c>
       <c r="C31" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="32">
@@ -7638,7 +7638,7 @@
         </is>
       </c>
       <c r="C32" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="33">
@@ -7653,7 +7653,7 @@
         </is>
       </c>
       <c r="C33" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="34">
@@ -7668,7 +7668,7 @@
         </is>
       </c>
       <c r="C34" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="35">
@@ -7683,7 +7683,7 @@
         </is>
       </c>
       <c r="C35" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="36">
@@ -7698,7 +7698,7 @@
         </is>
       </c>
       <c r="C36" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="37">
@@ -7713,7 +7713,7 @@
         </is>
       </c>
       <c r="C37" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="38">
@@ -7728,7 +7728,7 @@
         </is>
       </c>
       <c r="C38" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="39">
@@ -7743,7 +7743,7 @@
         </is>
       </c>
       <c r="C39" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="40">
@@ -7758,7 +7758,7 @@
         </is>
       </c>
       <c r="C40" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="41">
@@ -7773,7 +7773,7 @@
         </is>
       </c>
       <c r="C41" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="42">
@@ -7788,7 +7788,7 @@
         </is>
       </c>
       <c r="C42" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="43">
@@ -7803,7 +7803,7 @@
         </is>
       </c>
       <c r="C43" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="44">
@@ -7818,7 +7818,7 @@
         </is>
       </c>
       <c r="C44" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="45">
@@ -7833,7 +7833,7 @@
         </is>
       </c>
       <c r="C45" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="46">
@@ -7848,7 +7848,7 @@
         </is>
       </c>
       <c r="C46" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="47">
@@ -7863,7 +7863,7 @@
         </is>
       </c>
       <c r="C47" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="48">
@@ -7878,7 +7878,7 @@
         </is>
       </c>
       <c r="C48" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="49">
@@ -7893,7 +7893,7 @@
         </is>
       </c>
       <c r="C49" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="50">
@@ -7908,7 +7908,7 @@
         </is>
       </c>
       <c r="C50" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="51">
@@ -7923,7 +7923,7 @@
         </is>
       </c>
       <c r="C51" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="52">
@@ -7938,7 +7938,7 @@
         </is>
       </c>
       <c r="C52" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="53">
@@ -7953,7 +7953,7 @@
         </is>
       </c>
       <c r="C53" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="54">
@@ -7968,7 +7968,7 @@
         </is>
       </c>
       <c r="C54" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="55">
@@ -7983,7 +7983,7 @@
         </is>
       </c>
       <c r="C55" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="56">
@@ -7998,7 +7998,7 @@
         </is>
       </c>
       <c r="C56" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="57">
@@ -8013,7 +8013,7 @@
         </is>
       </c>
       <c r="C57" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="58">
@@ -8028,7 +8028,7 @@
         </is>
       </c>
       <c r="C58" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="59">
@@ -8043,7 +8043,7 @@
         </is>
       </c>
       <c r="C59" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="60">
@@ -8058,7 +8058,7 @@
         </is>
       </c>
       <c r="C60" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="61">
@@ -8073,7 +8073,7 @@
         </is>
       </c>
       <c r="C61" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="62">
@@ -8088,7 +8088,7 @@
         </is>
       </c>
       <c r="C62" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="63">
@@ -8103,7 +8103,7 @@
         </is>
       </c>
       <c r="C63" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="64">
@@ -8118,7 +8118,7 @@
         </is>
       </c>
       <c r="C64" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="65">
@@ -8133,7 +8133,7 @@
         </is>
       </c>
       <c r="C65" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="66">
@@ -8148,7 +8148,7 @@
         </is>
       </c>
       <c r="C66" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="67">
@@ -8163,7 +8163,7 @@
         </is>
       </c>
       <c r="C67" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="68">
@@ -8178,7 +8178,7 @@
         </is>
       </c>
       <c r="C68" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="69">
@@ -8193,7 +8193,7 @@
         </is>
       </c>
       <c r="C69" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="70">
@@ -8208,7 +8208,7 @@
         </is>
       </c>
       <c r="C70" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="71">
@@ -8223,7 +8223,7 @@
         </is>
       </c>
       <c r="C71" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="72">
@@ -8238,7 +8238,7 @@
         </is>
       </c>
       <c r="C72" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="73">
@@ -8253,7 +8253,7 @@
         </is>
       </c>
       <c r="C73" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="74">
@@ -8268,7 +8268,7 @@
         </is>
       </c>
       <c r="C74" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="75">
@@ -8283,7 +8283,7 @@
         </is>
       </c>
       <c r="C75" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="76">
@@ -8298,7 +8298,7 @@
         </is>
       </c>
       <c r="C76" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="77">
@@ -8313,7 +8313,7 @@
         </is>
       </c>
       <c r="C77" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="78">
@@ -8328,7 +8328,7 @@
         </is>
       </c>
       <c r="C78" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="79">
@@ -8343,7 +8343,7 @@
         </is>
       </c>
       <c r="C79" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="80">
@@ -8358,7 +8358,7 @@
         </is>
       </c>
       <c r="C80" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="81">
@@ -8373,7 +8373,7 @@
         </is>
       </c>
       <c r="C81" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="82">
@@ -8388,7 +8388,7 @@
         </is>
       </c>
       <c r="C82" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="83">
@@ -8403,7 +8403,7 @@
         </is>
       </c>
       <c r="C83" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="84">
@@ -8418,7 +8418,7 @@
         </is>
       </c>
       <c r="C84" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="85">
@@ -8433,7 +8433,7 @@
         </is>
       </c>
       <c r="C85" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="86">
@@ -8448,7 +8448,7 @@
         </is>
       </c>
       <c r="C86" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="87">
@@ -8463,7 +8463,7 @@
         </is>
       </c>
       <c r="C87" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="88">
@@ -8478,7 +8478,7 @@
         </is>
       </c>
       <c r="C88" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="89">
@@ -8493,7 +8493,7 @@
         </is>
       </c>
       <c r="C89" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="90">
@@ -8508,7 +8508,7 @@
         </is>
       </c>
       <c r="C90" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="91">
@@ -8523,7 +8523,7 @@
         </is>
       </c>
       <c r="C91" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="92">
@@ -8538,7 +8538,7 @@
         </is>
       </c>
       <c r="C92" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="93">
@@ -8553,7 +8553,7 @@
         </is>
       </c>
       <c r="C93" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="94">
@@ -8568,7 +8568,7 @@
         </is>
       </c>
       <c r="C94" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="95">
@@ -8583,7 +8583,7 @@
         </is>
       </c>
       <c r="C95" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="96">
@@ -8598,7 +8598,7 @@
         </is>
       </c>
       <c r="C96" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="97">
@@ -8613,7 +8613,7 @@
         </is>
       </c>
       <c r="C97" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="98">
@@ -8628,7 +8628,7 @@
         </is>
       </c>
       <c r="C98" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="99">
@@ -8643,7 +8643,7 @@
         </is>
       </c>
       <c r="C99" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="100">
@@ -8658,7 +8658,7 @@
         </is>
       </c>
       <c r="C100" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="101">
@@ -8673,7 +8673,7 @@
         </is>
       </c>
       <c r="C101" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="102">
@@ -8688,7 +8688,7 @@
         </is>
       </c>
       <c r="C102" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="103">
@@ -8703,7 +8703,7 @@
         </is>
       </c>
       <c r="C103" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="104">
@@ -8718,7 +8718,7 @@
         </is>
       </c>
       <c r="C104" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="105">
@@ -8733,7 +8733,7 @@
         </is>
       </c>
       <c r="C105" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="106">
@@ -8748,7 +8748,7 @@
         </is>
       </c>
       <c r="C106" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="107">
@@ -8763,7 +8763,7 @@
         </is>
       </c>
       <c r="C107" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="108">
@@ -8778,7 +8778,7 @@
         </is>
       </c>
       <c r="C108" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="109">
@@ -8793,7 +8793,7 @@
         </is>
       </c>
       <c r="C109" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="110">
@@ -8808,7 +8808,7 @@
         </is>
       </c>
       <c r="C110" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="111">
@@ -8823,7 +8823,7 @@
         </is>
       </c>
       <c r="C111" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="112">
@@ -8838,7 +8838,7 @@
         </is>
       </c>
       <c r="C112" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="113">
@@ -8853,7 +8853,7 @@
         </is>
       </c>
       <c r="C113" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>